<commit_message>
added water supply exceedance plots and some formatting
</commit_message>
<xml_diff>
--- a/inputs/water_supply_formulas.xlsx
+++ b/inputs/water_supply_formulas.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/fnufferrodriguez_usbr_gov/Documents/Desktop/eis-appendix-generation/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="11_F25DC773A252ABDACC10488381D843225BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25A7888C-1C23-448B-B446-B3CF6255FA94}"/>
+  <xr:revisionPtr revIDLastSave="238" documentId="11_F25DC773A252ABDACC10488381D843225BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFFD1ECC-9973-4663-8C7A-804D4731FEFB}"/>
   <bookViews>
-    <workbookView xWindow="-36885" yWindow="945" windowWidth="32115" windowHeight="18525" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-76920" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="annual" sheetId="1" r:id="rId1"/>
     <sheet name="final" sheetId="2" r:id="rId2"/>
+    <sheet name="exceedance" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -225,7 +226,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="285">
   <si>
     <t>Title</t>
   </si>
@@ -971,42 +972,24 @@
     <t>Total CVP North of Delta</t>
   </si>
   <si>
-    <t>Total CVP Ag and M&amp;I NOD</t>
-  </si>
-  <si>
     <t>Total SWP North of Delta</t>
   </si>
   <si>
-    <t>Total SWP Ag and M&amp;I NOD</t>
-  </si>
-  <si>
     <t>Total North of Delta</t>
   </si>
   <si>
-    <t>Total North of Delta Ag and M&amp;I Deliveries</t>
-  </si>
-  <si>
     <t>South of Delta</t>
   </si>
   <si>
     <t>Total CVP South of Delta</t>
   </si>
   <si>
-    <t>Total CVP Ag and M&amp;I SOD</t>
-  </si>
-  <si>
     <t>Total SWP South of Delta</t>
   </si>
   <si>
-    <t>Total SWP Ag and M&amp;I SOD</t>
-  </si>
-  <si>
     <t>Total South of Delta</t>
   </si>
   <si>
-    <t>Total South of Delta Ag and M&amp;I Deliveries</t>
-  </si>
-  <si>
     <t>Contract Delivery (annual average)</t>
   </si>
   <si>
@@ -1056,6 +1039,48 @@
   </si>
   <si>
     <t xml:space="preserve">(TAF/year) </t>
+  </si>
+  <si>
+    <t>CVP North of Delta Agricultural Water Service Contract Deliveries, Annual (Mar-Feb)</t>
+  </si>
+  <si>
+    <t>CVP South of Delta Agricultural Water Service Contract Deliveries, Annual (Mar-Feb)</t>
+  </si>
+  <si>
+    <t>CVP North of Delta M&amp;I Water Service Contract Deliveries, Annual (Mar-Feb)</t>
+  </si>
+  <si>
+    <t>CVP South of Delta M&amp;I Water Service Contract Deliveries, Annual (Mar-Feb)</t>
+  </si>
+  <si>
+    <t>Total SWP Deliveries, Annual (Jan-Dec)</t>
+  </si>
+  <si>
+    <t>Total SWP South of Delta Deliveries including Article 21 and 56, Annual (Jan-Dec)</t>
+  </si>
+  <si>
+    <t>SWP Table A Deliveries with Article 56, Annual (Jan-Dec)</t>
+  </si>
+  <si>
+    <t>SWP South of Delta Table A Deliveries with Article 56, Annual (Jan-Dec)</t>
+  </si>
+  <si>
+    <t>SWP Article 21 Deliveries, Annual (Jan-Dec)</t>
+  </si>
+  <si>
+    <t>Total Delta Exports, Annual (Oct-Sep)</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Total CVP Ag and M&amp;I</t>
+  </si>
+  <si>
+    <t>Total SWP Ag and M&amp;I</t>
+  </si>
+  <si>
+    <t>Total Ag and M&amp;I Deliveries</t>
   </si>
 </sst>
 </file>
@@ -1227,7 +1252,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1316,17 +1341,11 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1341,6 +1360,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -4071,51 +4104,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="40" t="s">
-        <v>271</v>
-      </c>
-      <c r="B1" s="40" t="s">
-        <v>272</v>
-      </c>
-      <c r="C1" s="40" t="s">
-        <v>273</v>
-      </c>
-      <c r="D1" s="40" t="s">
-        <v>275</v>
+      <c r="A1" s="38" t="s">
+        <v>265</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>266</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>267</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>269</v>
       </c>
       <c r="E1" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="45" t="s">
         <v>230</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D2" s="41" t="s">
-        <v>276</v>
-      </c>
-      <c r="E2" s="30" t="s">
+      <c r="C2" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="E2" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="F2" s="30" t="s">
+      <c r="F2" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="G2" s="30" t="s">
+      <c r="G2" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="30" t="s">
+      <c r="H2" s="44" t="s">
         <v>64</v>
       </c>
-      <c r="I2" s="30" t="s">
+      <c r="I2" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="J2" s="30" t="s">
+      <c r="J2" s="44" t="s">
         <v>68</v>
       </c>
       <c r="K2" s="30"/>
@@ -4142,15 +4175,15 @@
       <c r="AB2" s="31"/>
     </row>
     <row r="3" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="32"/>
-      <c r="B3" s="33" t="s">
+      <c r="A3" s="45"/>
+      <c r="B3" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="C3" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D3" s="41" t="s">
-        <v>276</v>
+      <c r="C3" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D3" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E3" s="30" t="s">
         <v>76</v>
@@ -4188,15 +4221,15 @@
       <c r="AB3" s="31"/>
     </row>
     <row r="4" spans="1:28" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="32"/>
-      <c r="B4" s="33" t="s">
+      <c r="A4" s="45"/>
+      <c r="B4" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="C4" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D4" s="41" t="s">
-        <v>276</v>
+      <c r="C4" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D4" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E4" s="30" t="s">
         <v>40</v>
@@ -4232,15 +4265,15 @@
       <c r="AB4" s="31"/>
     </row>
     <row r="5" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="32"/>
-      <c r="B5" s="33" t="s">
+      <c r="A5" s="45"/>
+      <c r="B5" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="C5" s="34" t="s">
-        <v>261</v>
-      </c>
-      <c r="D5" s="41" t="s">
-        <v>276</v>
+      <c r="C5" s="33" t="s">
+        <v>255</v>
+      </c>
+      <c r="D5" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E5" s="30" t="s">
         <v>6</v>
@@ -4276,15 +4309,15 @@
       <c r="AB5" s="31"/>
     </row>
     <row r="6" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="32"/>
-      <c r="B6" s="33" t="s">
+      <c r="A6" s="45"/>
+      <c r="B6" s="32" t="s">
         <v>234</v>
       </c>
-      <c r="C6" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D6" s="41" t="s">
-        <v>276</v>
+      <c r="C6" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E6" s="30" t="s">
         <v>193</v>
@@ -4322,15 +4355,15 @@
       <c r="AB6" s="31"/>
     </row>
     <row r="7" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="32"/>
-      <c r="B7" s="33" t="s">
+      <c r="A7" s="45"/>
+      <c r="B7" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C7" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D7" s="41" t="s">
-        <v>276</v>
+      <c r="C7" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E7" s="30" t="s">
         <v>136</v>
@@ -4362,17 +4395,17 @@
       <c r="AB7" s="31"/>
     </row>
     <row r="8" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="46" t="s">
         <v>236</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="C8" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D8" s="41" t="s">
-        <v>276</v>
+      <c r="C8" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E8" s="30" t="s">
         <v>70</v>
@@ -4406,15 +4439,15 @@
       <c r="AB8" s="31"/>
     </row>
     <row r="9" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="35"/>
-      <c r="B9" s="33" t="s">
+      <c r="A9" s="46"/>
+      <c r="B9" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="C9" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D9" s="41" t="s">
-        <v>276</v>
+      <c r="C9" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D9" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E9" s="30" t="s">
         <v>87</v>
@@ -4448,15 +4481,15 @@
       <c r="AB9" s="31"/>
     </row>
     <row r="10" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="35"/>
-      <c r="B10" s="33" t="s">
+      <c r="A10" s="46"/>
+      <c r="B10" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="C10" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D10" s="41" t="s">
-        <v>276</v>
+      <c r="C10" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D10" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E10" s="30" t="s">
         <v>55</v>
@@ -4486,15 +4519,15 @@
       <c r="AB10" s="31"/>
     </row>
     <row r="11" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="35"/>
-      <c r="B11" s="33" t="s">
+      <c r="A11" s="46"/>
+      <c r="B11" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="C11" s="34" t="s">
-        <v>262</v>
-      </c>
-      <c r="D11" s="41" t="s">
-        <v>276</v>
+      <c r="C11" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E11" s="30" t="s">
         <v>21</v>
@@ -4534,15 +4567,15 @@
       <c r="AB11" s="31"/>
     </row>
     <row r="12" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="35"/>
-      <c r="B12" s="33" t="s">
+      <c r="A12" s="46"/>
+      <c r="B12" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C12" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="D12" s="41" t="s">
-        <v>276</v>
+      <c r="C12" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E12" s="30" t="s">
         <v>114</v>
@@ -4572,17 +4605,17 @@
       <c r="AB12" s="31"/>
     </row>
     <row r="13" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="45" t="s">
         <v>239</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="C13" s="36" t="s">
-        <v>260</v>
-      </c>
-      <c r="D13" s="41" t="s">
-        <v>276</v>
+      <c r="C13" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="D13" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E13" s="30" t="s">
         <v>49</v>
@@ -4616,15 +4649,15 @@
       <c r="AB13" s="31"/>
     </row>
     <row r="14" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="32"/>
-      <c r="B14" s="33" t="s">
+      <c r="A14" s="45"/>
+      <c r="B14" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="C14" s="36" t="s">
-        <v>260</v>
-      </c>
-      <c r="D14" s="41" t="s">
-        <v>276</v>
+      <c r="C14" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="D14" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E14" s="30" t="s">
         <v>19</v>
@@ -4654,15 +4687,15 @@
       <c r="AB14" s="31"/>
     </row>
     <row r="15" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="32"/>
-      <c r="B15" s="33" t="s">
+      <c r="A15" s="45"/>
+      <c r="B15" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C15" s="34" t="s">
-        <v>264</v>
-      </c>
-      <c r="D15" s="41" t="s">
-        <v>276</v>
+      <c r="C15" s="33" t="s">
+        <v>258</v>
+      </c>
+      <c r="D15" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E15" s="30" t="s">
         <v>141</v>
@@ -4700,17 +4733,17 @@
       <c r="AB15" s="31"/>
     </row>
     <row r="16" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="35" t="s">
         <v>240</v>
       </c>
-      <c r="B16" s="33" t="s">
+      <c r="B16" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C16" s="36" t="s">
-        <v>265</v>
-      </c>
-      <c r="D16" s="41" t="s">
-        <v>276</v>
+      <c r="C16" s="34" t="s">
+        <v>259</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E16" s="30" t="s">
         <v>151</v>
@@ -4742,17 +4775,17 @@
       <c r="AB16" s="31"/>
     </row>
     <row r="17" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="35" t="s">
+      <c r="A17" s="46" t="s">
         <v>241</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="C17" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D17" s="41" t="s">
-        <v>276</v>
+      <c r="C17" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D17" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E17" s="30" t="s">
         <v>93</v>
@@ -4782,15 +4815,15 @@
       <c r="AB17" s="31"/>
     </row>
     <row r="18" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="35"/>
-      <c r="B18" s="33" t="s">
+      <c r="A18" s="46"/>
+      <c r="B18" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="C18" s="34" t="s">
-        <v>266</v>
-      </c>
-      <c r="D18" s="41" t="s">
-        <v>276</v>
+      <c r="C18" s="33" t="s">
+        <v>260</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E18" s="30" t="s">
         <v>32</v>
@@ -4826,15 +4859,15 @@
       <c r="AB18" s="31"/>
     </row>
     <row r="19" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="35"/>
-      <c r="B19" s="33" t="s">
+      <c r="A19" s="46"/>
+      <c r="B19" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C19" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D19" s="41" t="s">
-        <v>276</v>
+      <c r="C19" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D19" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E19" s="30" t="s">
         <v>155</v>
@@ -4864,15 +4897,15 @@
       <c r="AB19" s="31"/>
     </row>
     <row r="20" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="35"/>
-      <c r="B20" s="33" t="s">
+      <c r="A20" s="46"/>
+      <c r="B20" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C20" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="D20" s="41" t="s">
-        <v>276</v>
+      <c r="C20" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E20" s="30" t="s">
         <v>118</v>
@@ -4916,17 +4949,17 @@
       <c r="AB20" s="31"/>
     </row>
     <row r="21" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="35" t="s">
         <v>242</v>
       </c>
-      <c r="B21" s="33" t="s">
+      <c r="B21" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C21" s="36" t="s">
-        <v>267</v>
-      </c>
-      <c r="D21" s="41" t="s">
-        <v>276</v>
+      <c r="C21" s="34" t="s">
+        <v>261</v>
+      </c>
+      <c r="D21" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E21" s="30" t="s">
         <v>157</v>
@@ -4968,17 +5001,17 @@
       <c r="AB21" s="31"/>
     </row>
     <row r="22" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="32" t="s">
+      <c r="A22" s="45" t="s">
         <v>243</v>
       </c>
-      <c r="B22" s="33" t="s">
+      <c r="B22" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C22" s="34" t="s">
-        <v>264</v>
-      </c>
-      <c r="D22" s="41" t="s">
-        <v>276</v>
+      <c r="C22" s="33" t="s">
+        <v>258</v>
+      </c>
+      <c r="D22" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E22" s="30" t="s">
         <v>171</v>
@@ -5028,15 +5061,15 @@
       <c r="AB22" s="31"/>
     </row>
     <row r="23" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="32"/>
-      <c r="B23" s="33" t="s">
+      <c r="A23" s="45"/>
+      <c r="B23" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C23" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="D23" s="41" t="s">
-        <v>276</v>
+      <c r="C23" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="D23" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E23" s="30" t="s">
         <v>134</v>
@@ -5066,17 +5099,17 @@
       <c r="AB23" s="31"/>
     </row>
     <row r="24" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="37" t="s">
+      <c r="A24" s="35" t="s">
         <v>244</v>
       </c>
-      <c r="B24" s="33" t="s">
+      <c r="B24" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="C24" s="34" t="s">
-        <v>268</v>
-      </c>
-      <c r="D24" s="41" t="s">
-        <v>276</v>
+      <c r="C24" s="33" t="s">
+        <v>262</v>
+      </c>
+      <c r="D24" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -5104,17 +5137,17 @@
       <c r="AB24" s="31"/>
     </row>
     <row r="25" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="32" t="s">
+      <c r="A25" s="45" t="s">
         <v>246</v>
       </c>
-      <c r="B25" s="33" t="s">
+      <c r="B25" s="47" t="s">
         <v>233</v>
       </c>
-      <c r="C25" s="34" t="s">
-        <v>262</v>
-      </c>
-      <c r="D25" s="41" t="s">
-        <v>276</v>
+      <c r="C25" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="D25" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E25" s="30" t="s">
         <v>6</v>
@@ -5150,15 +5183,15 @@
       <c r="AB25" s="31"/>
     </row>
     <row r="26" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="32"/>
-      <c r="B26" s="33" t="s">
+      <c r="A26" s="45"/>
+      <c r="B26" s="47" t="s">
         <v>232</v>
       </c>
-      <c r="C26" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D26" s="41" t="s">
-        <v>276</v>
+      <c r="C26" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D26" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E26" s="30" t="s">
         <v>40</v>
@@ -5198,15 +5231,15 @@
       <c r="AB26" s="31"/>
     </row>
     <row r="27" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="32"/>
-      <c r="B27" s="33" t="s">
+      <c r="A27" s="45"/>
+      <c r="B27" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C27" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="D27" s="41" t="s">
-        <v>276</v>
+      <c r="C27" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="D27" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E27" s="30"/>
       <c r="F27" s="30"/>
@@ -5234,15 +5267,15 @@
       <c r="AB27" s="31"/>
     </row>
     <row r="28" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="32"/>
-      <c r="B28" s="33" t="s">
+      <c r="A28" s="45"/>
+      <c r="B28" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C28" s="34" t="s">
-        <v>264</v>
-      </c>
-      <c r="D28" s="41" t="s">
-        <v>276</v>
+      <c r="C28" s="33" t="s">
+        <v>258</v>
+      </c>
+      <c r="D28" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E28" s="30" t="s">
         <v>136</v>
@@ -5278,17 +5311,17 @@
       <c r="AB28" s="31"/>
     </row>
     <row r="29" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="35" t="s">
         <v>247</v>
       </c>
-      <c r="B29" s="33" t="s">
-        <v>248</v>
-      </c>
-      <c r="C29" s="34" t="s">
-        <v>269</v>
-      </c>
-      <c r="D29" s="41" t="s">
-        <v>276</v>
+      <c r="B29" s="32" t="s">
+        <v>282</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>263</v>
+      </c>
+      <c r="D29" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E29" s="31"/>
       <c r="F29" s="31"/>
@@ -5316,17 +5349,17 @@
       <c r="AB29" s="31"/>
     </row>
     <row r="30" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="37" t="s">
-        <v>249</v>
-      </c>
-      <c r="B30" s="33" t="s">
-        <v>250</v>
-      </c>
-      <c r="C30" s="34" t="s">
+      <c r="A30" s="35" t="s">
+        <v>248</v>
+      </c>
+      <c r="B30" s="32" t="s">
+        <v>283</v>
+      </c>
+      <c r="C30" s="33" t="s">
+        <v>264</v>
+      </c>
+      <c r="D30" s="39" t="s">
         <v>270</v>
-      </c>
-      <c r="D30" s="41" t="s">
-        <v>276</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -5354,17 +5387,17 @@
       <c r="AB30" s="31"/>
     </row>
     <row r="31" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="37" t="s">
-        <v>251</v>
-      </c>
-      <c r="B31" s="38" t="s">
-        <v>252</v>
-      </c>
-      <c r="C31" s="34" t="s">
-        <v>268</v>
-      </c>
-      <c r="D31" s="41" t="s">
-        <v>276</v>
+      <c r="A31" s="35" t="s">
+        <v>249</v>
+      </c>
+      <c r="B31" s="36" t="s">
+        <v>284</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>262</v>
+      </c>
+      <c r="D31" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -5392,17 +5425,17 @@
       <c r="AB31" s="31"/>
     </row>
     <row r="32" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="32" t="s">
-        <v>253</v>
-      </c>
-      <c r="B32" s="33" t="s">
+      <c r="A32" s="45" t="s">
+        <v>250</v>
+      </c>
+      <c r="B32" s="47" t="s">
         <v>233</v>
       </c>
-      <c r="C32" s="34" t="s">
-        <v>262</v>
-      </c>
-      <c r="D32" s="41" t="s">
-        <v>276</v>
+      <c r="C32" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="D32" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E32" s="30" t="s">
         <v>19</v>
@@ -5452,15 +5485,15 @@
       <c r="AB32" s="31"/>
     </row>
     <row r="33" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="32"/>
-      <c r="B33" s="33" t="s">
+      <c r="A33" s="45"/>
+      <c r="B33" s="47" t="s">
         <v>232</v>
       </c>
-      <c r="C33" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="D33" s="41" t="s">
-        <v>276</v>
+      <c r="C33" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D33" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E33" s="30" t="s">
         <v>53</v>
@@ -5492,15 +5525,15 @@
       <c r="AB33" s="31"/>
     </row>
     <row r="34" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="32"/>
-      <c r="B34" s="33" t="s">
+      <c r="A34" s="45"/>
+      <c r="B34" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C34" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="D34" s="41" t="s">
-        <v>276</v>
+      <c r="C34" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="D34" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E34" s="30" t="s">
         <v>134</v>
@@ -5530,15 +5563,15 @@
       <c r="AB34" s="31"/>
     </row>
     <row r="35" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="32"/>
-      <c r="B35" s="33" t="s">
+      <c r="A35" s="45"/>
+      <c r="B35" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C35" s="34" t="s">
-        <v>264</v>
-      </c>
-      <c r="D35" s="41" t="s">
-        <v>276</v>
+      <c r="C35" s="33" t="s">
+        <v>258</v>
+      </c>
+      <c r="D35" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E35" s="30" t="s">
         <v>145</v>
@@ -5614,17 +5647,17 @@
       </c>
     </row>
     <row r="36" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="37" t="s">
-        <v>254</v>
-      </c>
-      <c r="B36" s="33" t="s">
-        <v>255</v>
-      </c>
-      <c r="C36" s="34" t="s">
-        <v>269</v>
-      </c>
-      <c r="D36" s="41" t="s">
-        <v>276</v>
+      <c r="A36" s="35" t="s">
+        <v>251</v>
+      </c>
+      <c r="B36" s="32" t="s">
+        <v>282</v>
+      </c>
+      <c r="C36" s="33" t="s">
+        <v>263</v>
+      </c>
+      <c r="D36" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -5652,17 +5685,17 @@
       <c r="AB36" s="31"/>
     </row>
     <row r="37" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="39" t="s">
-        <v>256</v>
-      </c>
-      <c r="B37" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="C37" s="34" t="s">
+      <c r="A37" s="37" t="s">
+        <v>252</v>
+      </c>
+      <c r="B37" s="32" t="s">
+        <v>283</v>
+      </c>
+      <c r="C37" s="33" t="s">
+        <v>264</v>
+      </c>
+      <c r="D37" s="39" t="s">
         <v>270</v>
-      </c>
-      <c r="D37" s="41" t="s">
-        <v>276</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -5690,17 +5723,17 @@
       <c r="AB37" s="31"/>
     </row>
     <row r="38" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="37" t="s">
-        <v>258</v>
-      </c>
-      <c r="B38" s="38" t="s">
-        <v>259</v>
-      </c>
-      <c r="C38" s="34" t="s">
-        <v>268</v>
-      </c>
-      <c r="D38" s="41" t="s">
-        <v>276</v>
+      <c r="A38" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="B38" s="36" t="s">
+        <v>284</v>
+      </c>
+      <c r="C38" s="33" t="s">
+        <v>262</v>
+      </c>
+      <c r="D38" s="39" t="s">
+        <v>270</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -5851,4 +5884,716 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1186BE7D-212F-4787-917F-2183B0DA8701}">
+  <dimension ref="A1:AR11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="73" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="38" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="2" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="42" t="s">
+        <v>271</v>
+      </c>
+      <c r="B2" s="40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="41"/>
+      <c r="R2" s="41"/>
+      <c r="S2" s="41"/>
+      <c r="T2" s="41"/>
+      <c r="U2" s="41"/>
+      <c r="V2" s="41"/>
+      <c r="W2" s="41"/>
+      <c r="X2" s="41"/>
+      <c r="Y2" s="41"/>
+      <c r="Z2" s="41"/>
+      <c r="AA2" s="41"/>
+      <c r="AB2" s="41"/>
+      <c r="AC2" s="41"/>
+      <c r="AD2" s="41"/>
+      <c r="AE2" s="41"/>
+      <c r="AF2" s="41"/>
+      <c r="AG2" s="41"/>
+      <c r="AH2" s="41"/>
+      <c r="AI2" s="41"/>
+      <c r="AJ2" s="41"/>
+      <c r="AK2" s="41"/>
+      <c r="AL2" s="41"/>
+      <c r="AM2" s="41"/>
+      <c r="AN2" s="41"/>
+      <c r="AO2" s="41"/>
+      <c r="AP2" s="41"/>
+      <c r="AQ2" s="41"/>
+      <c r="AR2" s="41"/>
+    </row>
+    <row r="3" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="42" t="s">
+        <v>272</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="40" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="40" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="40" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" s="41"/>
+      <c r="N3" s="41"/>
+      <c r="O3" s="41"/>
+      <c r="P3" s="41"/>
+      <c r="Q3" s="41"/>
+      <c r="R3" s="41"/>
+      <c r="S3" s="41"/>
+      <c r="T3" s="41"/>
+      <c r="U3" s="41"/>
+      <c r="V3" s="41"/>
+      <c r="W3" s="41"/>
+      <c r="X3" s="41"/>
+      <c r="Y3" s="41"/>
+      <c r="Z3" s="41"/>
+      <c r="AA3" s="41"/>
+      <c r="AB3" s="41"/>
+      <c r="AC3" s="41"/>
+      <c r="AD3" s="41"/>
+      <c r="AE3" s="41"/>
+      <c r="AF3" s="41"/>
+      <c r="AG3" s="41"/>
+      <c r="AH3" s="41"/>
+      <c r="AI3" s="41"/>
+      <c r="AJ3" s="41"/>
+      <c r="AK3" s="41"/>
+      <c r="AL3" s="41"/>
+      <c r="AM3" s="41"/>
+      <c r="AN3" s="41"/>
+      <c r="AO3" s="41"/>
+      <c r="AP3" s="41"/>
+      <c r="AQ3" s="41"/>
+      <c r="AR3" s="41"/>
+    </row>
+    <row r="4" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="B4" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="41"/>
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="41"/>
+      <c r="V4" s="41"/>
+      <c r="W4" s="41"/>
+      <c r="X4" s="41"/>
+      <c r="Y4" s="41"/>
+      <c r="Z4" s="41"/>
+      <c r="AA4" s="41"/>
+      <c r="AB4" s="41"/>
+      <c r="AC4" s="41"/>
+      <c r="AD4" s="41"/>
+      <c r="AE4" s="41"/>
+      <c r="AF4" s="41"/>
+      <c r="AG4" s="41"/>
+      <c r="AH4" s="41"/>
+      <c r="AI4" s="41"/>
+      <c r="AJ4" s="41"/>
+      <c r="AK4" s="41"/>
+      <c r="AL4" s="41"/>
+      <c r="AM4" s="41"/>
+      <c r="AN4" s="41"/>
+      <c r="AO4" s="41"/>
+      <c r="AP4" s="41"/>
+      <c r="AQ4" s="41"/>
+      <c r="AR4" s="41"/>
+    </row>
+    <row r="5" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="42" t="s">
+        <v>274</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="41"/>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="41"/>
+      <c r="R5" s="41"/>
+      <c r="S5" s="41"/>
+      <c r="T5" s="41"/>
+      <c r="U5" s="41"/>
+      <c r="V5" s="41"/>
+      <c r="W5" s="41"/>
+      <c r="X5" s="41"/>
+      <c r="Y5" s="41"/>
+      <c r="Z5" s="41"/>
+      <c r="AA5" s="41"/>
+      <c r="AB5" s="41"/>
+      <c r="AC5" s="41"/>
+      <c r="AD5" s="41"/>
+      <c r="AE5" s="41"/>
+      <c r="AF5" s="41"/>
+      <c r="AG5" s="41"/>
+      <c r="AH5" s="41"/>
+      <c r="AI5" s="41"/>
+      <c r="AJ5" s="41"/>
+      <c r="AK5" s="41"/>
+      <c r="AL5" s="41"/>
+      <c r="AM5" s="41"/>
+      <c r="AN5" s="41"/>
+      <c r="AO5" s="41"/>
+      <c r="AP5" s="41"/>
+      <c r="AQ5" s="41"/>
+      <c r="AR5" s="41"/>
+    </row>
+    <row r="6" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="42" t="s">
+        <v>275</v>
+      </c>
+      <c r="B6" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="E6" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="G6" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="H6" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="I6" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="J6" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="K6" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="L6" s="40" t="s">
+        <v>136</v>
+      </c>
+      <c r="M6" s="40" t="s">
+        <v>139</v>
+      </c>
+      <c r="N6" s="40" t="s">
+        <v>141</v>
+      </c>
+      <c r="O6" s="40" t="s">
+        <v>143</v>
+      </c>
+      <c r="P6" s="40" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q6" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="R6" s="40" t="s">
+        <v>149</v>
+      </c>
+      <c r="S6" s="40" t="s">
+        <v>151</v>
+      </c>
+      <c r="T6" s="40" t="s">
+        <v>153</v>
+      </c>
+      <c r="U6" s="40" t="s">
+        <v>155</v>
+      </c>
+      <c r="V6" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="W6" s="40" t="s">
+        <v>159</v>
+      </c>
+      <c r="X6" s="40" t="s">
+        <v>161</v>
+      </c>
+      <c r="Y6" s="40" t="s">
+        <v>163</v>
+      </c>
+      <c r="Z6" s="40" t="s">
+        <v>165</v>
+      </c>
+      <c r="AA6" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB6" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="AC6" s="40" t="s">
+        <v>171</v>
+      </c>
+      <c r="AD6" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="AE6" s="40" t="s">
+        <v>175</v>
+      </c>
+      <c r="AF6" s="40" t="s">
+        <v>177</v>
+      </c>
+      <c r="AG6" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="AH6" s="40" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI6" s="40" t="s">
+        <v>183</v>
+      </c>
+      <c r="AJ6" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="AK6" s="40" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL6" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="AM6" s="40" t="s">
+        <v>191</v>
+      </c>
+      <c r="AN6" s="40" t="s">
+        <v>193</v>
+      </c>
+      <c r="AO6" s="40" t="s">
+        <v>196</v>
+      </c>
+      <c r="AP6" s="40" t="s">
+        <v>198</v>
+      </c>
+      <c r="AQ6" s="40" t="s">
+        <v>200</v>
+      </c>
+      <c r="AR6" s="40" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="43" t="s">
+        <v>276</v>
+      </c>
+      <c r="B7" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C7" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="E7" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="G7" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="H7" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="I7" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="J7" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="K7" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="L7" s="40" t="s">
+        <v>145</v>
+      </c>
+      <c r="M7" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="N7" s="40" t="s">
+        <v>149</v>
+      </c>
+      <c r="O7" s="40" t="s">
+        <v>151</v>
+      </c>
+      <c r="P7" s="40" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q7" s="40" t="s">
+        <v>155</v>
+      </c>
+      <c r="R7" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="S7" s="40" t="s">
+        <v>159</v>
+      </c>
+      <c r="T7" s="40" t="s">
+        <v>161</v>
+      </c>
+      <c r="U7" s="40" t="s">
+        <v>163</v>
+      </c>
+      <c r="V7" s="40" t="s">
+        <v>165</v>
+      </c>
+      <c r="W7" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="X7" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="Y7" s="40" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z7" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="AA7" s="40" t="s">
+        <v>175</v>
+      </c>
+      <c r="AB7" s="40" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC7" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="AD7" s="40" t="s">
+        <v>181</v>
+      </c>
+      <c r="AE7" s="40" t="s">
+        <v>183</v>
+      </c>
+      <c r="AF7" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="AG7" s="40" t="s">
+        <v>187</v>
+      </c>
+      <c r="AH7" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="AI7" s="40" t="s">
+        <v>191</v>
+      </c>
+      <c r="AJ7" s="41"/>
+      <c r="AK7" s="41"/>
+      <c r="AL7" s="41"/>
+      <c r="AM7" s="41"/>
+      <c r="AN7" s="41"/>
+      <c r="AO7" s="41"/>
+      <c r="AP7" s="41"/>
+      <c r="AQ7" s="41"/>
+      <c r="AR7" s="41"/>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="43" t="s">
+        <v>277</v>
+      </c>
+      <c r="B8" s="40" t="s">
+        <v>215</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>217</v>
+      </c>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="41"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="41"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="41"/>
+      <c r="O8" s="41"/>
+      <c r="P8" s="41"/>
+      <c r="Q8" s="41"/>
+      <c r="R8" s="41"/>
+      <c r="S8" s="41"/>
+      <c r="T8" s="41"/>
+      <c r="U8" s="41"/>
+      <c r="V8" s="41"/>
+      <c r="W8" s="41"/>
+      <c r="X8" s="41"/>
+      <c r="Y8" s="41"/>
+      <c r="Z8" s="41"/>
+      <c r="AA8" s="41"/>
+      <c r="AB8" s="41"/>
+      <c r="AC8" s="41"/>
+      <c r="AD8" s="41"/>
+      <c r="AE8" s="41"/>
+      <c r="AF8" s="41"/>
+      <c r="AG8" s="41"/>
+      <c r="AH8" s="41"/>
+      <c r="AI8" s="41"/>
+      <c r="AJ8" s="41"/>
+      <c r="AK8" s="41"/>
+      <c r="AL8" s="41"/>
+      <c r="AM8" s="41"/>
+      <c r="AN8" s="41"/>
+      <c r="AO8" s="41"/>
+      <c r="AP8" s="41"/>
+      <c r="AQ8" s="41"/>
+      <c r="AR8" s="41"/>
+    </row>
+    <row r="9" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="43" t="s">
+        <v>278</v>
+      </c>
+      <c r="B9" s="40" t="s">
+        <v>215</v>
+      </c>
+      <c r="C9" s="40" t="s">
+        <v>217</v>
+      </c>
+      <c r="D9" s="41" t="s">
+        <v>221</v>
+      </c>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="41"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="41"/>
+      <c r="M9" s="41"/>
+      <c r="N9" s="41"/>
+      <c r="O9" s="41"/>
+      <c r="P9" s="41"/>
+      <c r="Q9" s="41"/>
+      <c r="R9" s="41"/>
+      <c r="S9" s="41"/>
+      <c r="T9" s="41"/>
+      <c r="U9" s="41"/>
+      <c r="V9" s="41"/>
+      <c r="W9" s="41"/>
+      <c r="X9" s="41"/>
+      <c r="Y9" s="41"/>
+      <c r="Z9" s="41"/>
+      <c r="AA9" s="41"/>
+      <c r="AB9" s="41"/>
+      <c r="AC9" s="41"/>
+      <c r="AD9" s="41"/>
+      <c r="AE9" s="41"/>
+      <c r="AF9" s="41"/>
+      <c r="AG9" s="41"/>
+      <c r="AH9" s="41"/>
+      <c r="AI9" s="41"/>
+      <c r="AJ9" s="41"/>
+      <c r="AK9" s="41"/>
+      <c r="AL9" s="41"/>
+      <c r="AM9" s="41"/>
+      <c r="AN9" s="41"/>
+      <c r="AO9" s="41"/>
+      <c r="AP9" s="41"/>
+      <c r="AQ9" s="41"/>
+      <c r="AR9" s="41"/>
+    </row>
+    <row r="10" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="43" t="s">
+        <v>279</v>
+      </c>
+      <c r="B10" s="40" t="s">
+        <v>219</v>
+      </c>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="41"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="41"/>
+      <c r="P10" s="41"/>
+      <c r="Q10" s="41"/>
+      <c r="R10" s="41"/>
+      <c r="S10" s="41"/>
+      <c r="T10" s="41"/>
+      <c r="U10" s="41"/>
+      <c r="V10" s="41"/>
+      <c r="W10" s="41"/>
+      <c r="X10" s="41"/>
+      <c r="Y10" s="41"/>
+      <c r="Z10" s="41"/>
+      <c r="AA10" s="41"/>
+      <c r="AB10" s="41"/>
+      <c r="AC10" s="41"/>
+      <c r="AD10" s="41"/>
+      <c r="AE10" s="41"/>
+      <c r="AF10" s="41"/>
+      <c r="AG10" s="41"/>
+      <c r="AH10" s="41"/>
+      <c r="AI10" s="41"/>
+      <c r="AJ10" s="41"/>
+      <c r="AK10" s="41"/>
+      <c r="AL10" s="41"/>
+      <c r="AM10" s="41"/>
+      <c r="AN10" s="41"/>
+      <c r="AO10" s="41"/>
+      <c r="AP10" s="41"/>
+      <c r="AQ10" s="41"/>
+      <c r="AR10" s="41"/>
+    </row>
+    <row r="11" spans="1:44" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="43" t="s">
+        <v>280</v>
+      </c>
+      <c r="B11" s="40" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="41"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+      <c r="M11" s="41"/>
+      <c r="N11" s="41"/>
+      <c r="O11" s="41"/>
+      <c r="P11" s="41"/>
+      <c r="Q11" s="41"/>
+      <c r="R11" s="41"/>
+      <c r="S11" s="41"/>
+      <c r="T11" s="41"/>
+      <c r="U11" s="41"/>
+      <c r="V11" s="41"/>
+      <c r="W11" s="41"/>
+      <c r="X11" s="41"/>
+      <c r="Y11" s="41"/>
+      <c r="Z11" s="41"/>
+      <c r="AA11" s="41"/>
+      <c r="AB11" s="41"/>
+      <c r="AC11" s="41"/>
+      <c r="AD11" s="41"/>
+      <c r="AE11" s="41"/>
+      <c r="AF11" s="41"/>
+      <c r="AG11" s="41"/>
+      <c r="AH11" s="41"/>
+      <c r="AI11" s="41"/>
+      <c r="AJ11" s="41"/>
+      <c r="AK11" s="41"/>
+      <c r="AL11" s="41"/>
+      <c r="AM11" s="41"/>
+      <c r="AN11" s="41"/>
+      <c r="AO11" s="41"/>
+      <c r="AP11" s="41"/>
+      <c r="AQ11" s="41"/>
+      <c r="AR11" s="41"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added in remaining steps for full water quality compliance appendix
</commit_message>
<xml_diff>
--- a/inputs/water_supply_formulas.xlsx
+++ b/inputs/water_supply_formulas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/fnufferrodriguez_usbr_gov/Documents/Desktop/eis-appendix-generation/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="265" documentId="11_F25DC773A252ABDACC10488381D843225BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE97C42A-C556-4E79-8592-7E9166B4DD35}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="11_F25DC773A252ABDACC10488381D843225BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBB79A27-40F6-4B64-803B-F9D08AFD795D}"/>
   <bookViews>
-    <workbookView xWindow="-28230" yWindow="4065" windowWidth="17100" windowHeight="16050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="20625" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="annual" sheetId="1" r:id="rId1"/>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1109" uniqueCount="286">
   <si>
     <t>Title</t>
   </si>
@@ -1084,33 +1084,6 @@
   </si>
   <si>
     <t>-SWP Table A NOD Deliveries</t>
-  </si>
-  <si>
-    <t>SWP_FRSA</t>
-  </si>
-  <si>
-    <t>DEL_CVP_PSC_N</t>
-  </si>
-  <si>
-    <t>DEL_CVP_PRF_N</t>
-  </si>
-  <si>
-    <t>DEL_CVP_PMI_N_WAMER</t>
-  </si>
-  <si>
-    <t>DEL_CVP_PAG_N</t>
-  </si>
-  <si>
-    <t>DEL_CVP_PEX_S</t>
-  </si>
-  <si>
-    <t>DEL_CVP_PRF_S</t>
-  </si>
-  <si>
-    <t>DEL_CVP_PMI_S</t>
-  </si>
-  <si>
-    <t>DEL_CVP_PAG_S</t>
   </si>
 </sst>
 </file>
@@ -1192,7 +1165,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1221,12 +1194,6 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA9D08E"/>
-        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -1365,13 +1332,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1397,21 +1365,20 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1770,7 +1737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="3" max="3" width="148.3671875" customWidth="1"/>
@@ -4122,186 +4089,6 @@
         <v>12</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A103" s="45" t="s">
-        <v>287</v>
-      </c>
-      <c r="C103" s="45" t="s">
-        <v>287</v>
-      </c>
-      <c r="D103" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F103" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G103" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A104" s="46" t="s">
-        <v>288</v>
-      </c>
-      <c r="C104" s="46" t="s">
-        <v>288</v>
-      </c>
-      <c r="D104" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E104" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F104" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G104" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A105" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="C105" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="D105" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E105" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F105" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G105" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A106" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="C106" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="D106" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E106" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F106" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G106" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A107" s="46" t="s">
-        <v>286</v>
-      </c>
-      <c r="C107" s="46" t="s">
-        <v>286</v>
-      </c>
-      <c r="D107" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E107" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F107" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G107" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A108" s="46" t="s">
-        <v>291</v>
-      </c>
-      <c r="C108" s="46" t="s">
-        <v>291</v>
-      </c>
-      <c r="D108" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E108" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F108" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G108" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A109" s="46" t="s">
-        <v>292</v>
-      </c>
-      <c r="C109" s="46" t="s">
-        <v>292</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E109" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F109" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G109" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A110" s="46" t="s">
-        <v>293</v>
-      </c>
-      <c r="C110" s="46" t="s">
-        <v>293</v>
-      </c>
-      <c r="D110" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E110" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F110" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G110" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A111" s="46" t="s">
-        <v>294</v>
-      </c>
-      <c r="C111" s="46" t="s">
-        <v>294</v>
-      </c>
-      <c r="D111" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E111" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F111" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G111" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -4310,10 +4097,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9C56A8D-8685-46A1-B439-8B094C2DFA58}">
-  <dimension ref="A1:AB61"/>
+  <dimension ref="A1:AB75"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="47.578125" customWidth="1"/>
+    <col min="1" max="1" width="36.5234375" customWidth="1"/>
     <col min="2" max="2" width="27.05078125" customWidth="1"/>
     <col min="3" max="3" width="40.05078125" customWidth="1"/>
     <col min="4" max="4" width="15.15625" customWidth="1"/>
@@ -4321,16 +4108,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>265</v>
       </c>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="38" t="s">
         <v>266</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="C1" s="38" t="s">
         <v>267</v>
       </c>
-      <c r="D1" s="37" t="s">
+      <c r="D1" s="38" t="s">
         <v>269</v>
       </c>
       <c r="E1" t="s">
@@ -4338,1623 +4125,1769 @@
       </c>
     </row>
     <row r="2" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="46" t="s">
         <v>230</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E2" s="45" t="s">
-        <v>287</v>
-      </c>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="30"/>
-      <c r="T2" s="30"/>
-      <c r="U2" s="30"/>
-      <c r="V2" s="30"/>
-      <c r="W2" s="30"/>
-      <c r="X2" s="30"/>
-      <c r="Y2" s="30"/>
-      <c r="Z2" s="30"/>
-      <c r="AA2" s="30"/>
-      <c r="AB2" s="30"/>
+      <c r="E2" s="44" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" s="44" t="s">
+        <v>64</v>
+      </c>
+      <c r="I2" s="44" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="31"/>
+      <c r="S2" s="31"/>
+      <c r="T2" s="31"/>
+      <c r="U2" s="31"/>
+      <c r="V2" s="31"/>
+      <c r="W2" s="31"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="31"/>
+      <c r="Z2" s="31"/>
+      <c r="AA2" s="31"/>
+      <c r="AB2" s="31"/>
     </row>
     <row r="3" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="47"/>
-      <c r="B3" s="31" t="s">
+      <c r="A3" s="46"/>
+      <c r="B3" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E3" s="46" t="s">
-        <v>288</v>
-      </c>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="30"/>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="30"/>
-      <c r="R3" s="30"/>
-      <c r="S3" s="30"/>
-      <c r="T3" s="30"/>
-      <c r="U3" s="30"/>
-      <c r="V3" s="30"/>
-      <c r="W3" s="30"/>
-      <c r="X3" s="30"/>
-      <c r="Y3" s="30"/>
-      <c r="Z3" s="30"/>
-      <c r="AA3" s="30"/>
-      <c r="AB3" s="30"/>
+      <c r="E3" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="H3" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="31"/>
+      <c r="T3" s="31"/>
+      <c r="U3" s="31"/>
+      <c r="V3" s="31"/>
+      <c r="W3" s="31"/>
+      <c r="X3" s="31"/>
+      <c r="Y3" s="31"/>
+      <c r="Z3" s="31"/>
+      <c r="AA3" s="31"/>
+      <c r="AB3" s="31"/>
     </row>
     <row r="4" spans="1:28" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="47"/>
-      <c r="B4" s="31" t="s">
+      <c r="A4" s="46"/>
+      <c r="B4" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E4" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
-      <c r="O4" s="30"/>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="30"/>
-      <c r="R4" s="30"/>
-      <c r="S4" s="30"/>
-      <c r="T4" s="30"/>
-      <c r="U4" s="30"/>
-      <c r="V4" s="30"/>
-      <c r="W4" s="30"/>
-      <c r="X4" s="30"/>
-      <c r="Y4" s="30"/>
-      <c r="Z4" s="30"/>
-      <c r="AA4" s="30"/>
-      <c r="AB4" s="30"/>
+      <c r="E4" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="31"/>
+      <c r="R4" s="31"/>
+      <c r="S4" s="31"/>
+      <c r="T4" s="31"/>
+      <c r="U4" s="31"/>
+      <c r="V4" s="31"/>
+      <c r="W4" s="31"/>
+      <c r="X4" s="31"/>
+      <c r="Y4" s="31"/>
+      <c r="Z4" s="31"/>
+      <c r="AA4" s="31"/>
+      <c r="AB4" s="31"/>
     </row>
     <row r="5" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="47"/>
-      <c r="B5" s="31" t="s">
+      <c r="A5" s="46"/>
+      <c r="B5" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="33" t="s">
         <v>255</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E5" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30"/>
-      <c r="U5" s="30"/>
-      <c r="V5" s="30"/>
-      <c r="W5" s="30"/>
-      <c r="X5" s="30"/>
-      <c r="Y5" s="30"/>
-      <c r="Z5" s="30"/>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="30"/>
+      <c r="E5" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="31"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="31"/>
+      <c r="W5" s="31"/>
+      <c r="X5" s="31"/>
+      <c r="Y5" s="31"/>
+      <c r="Z5" s="31"/>
+      <c r="AA5" s="31"/>
+      <c r="AB5" s="31"/>
     </row>
     <row r="6" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="47"/>
-      <c r="B6" s="31" t="s">
+      <c r="A6" s="46"/>
+      <c r="B6" s="32" t="s">
         <v>234</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="D6" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E6" s="46" t="s">
-        <v>286</v>
-      </c>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="30"/>
-      <c r="K6" s="30"/>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="30"/>
-      <c r="O6" s="30"/>
-      <c r="P6" s="30"/>
-      <c r="Q6" s="30"/>
-      <c r="R6" s="30"/>
-      <c r="S6" s="30"/>
-      <c r="T6" s="30"/>
-      <c r="U6" s="30"/>
-      <c r="V6" s="30"/>
-      <c r="W6" s="30"/>
-      <c r="X6" s="30"/>
-      <c r="Y6" s="30"/>
-      <c r="Z6" s="30"/>
-      <c r="AA6" s="30"/>
-      <c r="AB6" s="30"/>
+      <c r="E6" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="G6" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="I6" s="30" t="s">
+        <v>202</v>
+      </c>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
+      <c r="O6" s="31"/>
+      <c r="P6" s="31"/>
+      <c r="Q6" s="31"/>
+      <c r="R6" s="31"/>
+      <c r="S6" s="31"/>
+      <c r="T6" s="31"/>
+      <c r="U6" s="31"/>
+      <c r="V6" s="31"/>
+      <c r="W6" s="31"/>
+      <c r="X6" s="31"/>
+      <c r="Y6" s="31"/>
+      <c r="Z6" s="31"/>
+      <c r="AA6" s="31"/>
+      <c r="AB6" s="31"/>
     </row>
     <row r="7" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="47"/>
-      <c r="B7" s="31" t="s">
+      <c r="A7" s="46"/>
+      <c r="B7" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D7" s="38" t="s">
+      <c r="D7" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="30" t="s">
         <v>136</v>
       </c>
-      <c r="F7" s="29" t="s">
+      <c r="F7" s="30" t="s">
         <v>139</v>
       </c>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="30"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="30"/>
-      <c r="O7" s="30"/>
-      <c r="P7" s="30"/>
-      <c r="Q7" s="30"/>
-      <c r="R7" s="30"/>
-      <c r="S7" s="30"/>
-      <c r="T7" s="30"/>
-      <c r="U7" s="30"/>
-      <c r="V7" s="30"/>
-      <c r="W7" s="30"/>
-      <c r="X7" s="30"/>
-      <c r="Y7" s="30"/>
-      <c r="Z7" s="30"/>
-      <c r="AA7" s="30"/>
-      <c r="AB7" s="30"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="31"/>
+      <c r="L7" s="31"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="31"/>
+      <c r="O7" s="31"/>
+      <c r="P7" s="31"/>
+      <c r="Q7" s="31"/>
+      <c r="R7" s="31"/>
+      <c r="S7" s="31"/>
+      <c r="T7" s="31"/>
+      <c r="U7" s="31"/>
+      <c r="V7" s="31"/>
+      <c r="W7" s="31"/>
+      <c r="X7" s="31"/>
+      <c r="Y7" s="31"/>
+      <c r="Z7" s="31"/>
+      <c r="AA7" s="31"/>
+      <c r="AB7" s="31"/>
     </row>
     <row r="8" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="47" t="s">
         <v>236</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E8" s="46" t="s">
-        <v>291</v>
-      </c>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="30"/>
-      <c r="N8" s="30"/>
-      <c r="O8" s="30"/>
-      <c r="P8" s="30"/>
-      <c r="Q8" s="30"/>
-      <c r="R8" s="30"/>
-      <c r="S8" s="30"/>
-      <c r="T8" s="30"/>
-      <c r="U8" s="30"/>
-      <c r="V8" s="30"/>
-      <c r="W8" s="30"/>
-      <c r="X8" s="30"/>
-      <c r="Y8" s="30"/>
-      <c r="Z8" s="30"/>
-      <c r="AA8" s="30"/>
-      <c r="AB8" s="30"/>
+      <c r="E8" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="31"/>
+      <c r="L8" s="31"/>
+      <c r="M8" s="31"/>
+      <c r="N8" s="31"/>
+      <c r="O8" s="31"/>
+      <c r="P8" s="31"/>
+      <c r="Q8" s="31"/>
+      <c r="R8" s="31"/>
+      <c r="S8" s="31"/>
+      <c r="T8" s="31"/>
+      <c r="U8" s="31"/>
+      <c r="V8" s="31"/>
+      <c r="W8" s="31"/>
+      <c r="X8" s="31"/>
+      <c r="Y8" s="31"/>
+      <c r="Z8" s="31"/>
+      <c r="AA8" s="31"/>
+      <c r="AB8" s="31"/>
     </row>
     <row r="9" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="48"/>
-      <c r="B9" s="31" t="s">
+      <c r="A9" s="47"/>
+      <c r="B9" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E9" s="46" t="s">
-        <v>292</v>
-      </c>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
-      <c r="P9" s="30"/>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
-      <c r="S9" s="30"/>
-      <c r="T9" s="30"/>
-      <c r="U9" s="30"/>
-      <c r="V9" s="30"/>
-      <c r="W9" s="30"/>
-      <c r="X9" s="30"/>
-      <c r="Y9" s="30"/>
-      <c r="Z9" s="30"/>
-      <c r="AA9" s="30"/>
-      <c r="AB9" s="30"/>
+      <c r="E9" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="31"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="31"/>
+      <c r="R9" s="31"/>
+      <c r="S9" s="31"/>
+      <c r="T9" s="31"/>
+      <c r="U9" s="31"/>
+      <c r="V9" s="31"/>
+      <c r="W9" s="31"/>
+      <c r="X9" s="31"/>
+      <c r="Y9" s="31"/>
+      <c r="Z9" s="31"/>
+      <c r="AA9" s="31"/>
+      <c r="AB9" s="31"/>
     </row>
     <row r="10" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="48"/>
-      <c r="B10" s="31" t="s">
+      <c r="A10" s="47"/>
+      <c r="B10" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D10" s="38" t="s">
+      <c r="D10" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E10" s="46" t="s">
-        <v>293</v>
-      </c>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="30"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="30"/>
-      <c r="P10" s="30"/>
-      <c r="Q10" s="30"/>
-      <c r="R10" s="30"/>
-      <c r="S10" s="30"/>
-      <c r="T10" s="30"/>
-      <c r="U10" s="30"/>
-      <c r="V10" s="30"/>
-      <c r="W10" s="30"/>
-      <c r="X10" s="30"/>
-      <c r="Y10" s="30"/>
-      <c r="Z10" s="30"/>
-      <c r="AA10" s="30"/>
-      <c r="AB10" s="30"/>
+      <c r="E10" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="31"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
+      <c r="O10" s="31"/>
+      <c r="P10" s="31"/>
+      <c r="Q10" s="31"/>
+      <c r="R10" s="31"/>
+      <c r="S10" s="31"/>
+      <c r="T10" s="31"/>
+      <c r="U10" s="31"/>
+      <c r="V10" s="31"/>
+      <c r="W10" s="31"/>
+      <c r="X10" s="31"/>
+      <c r="Y10" s="31"/>
+      <c r="Z10" s="31"/>
+      <c r="AA10" s="31"/>
+      <c r="AB10" s="31"/>
     </row>
     <row r="11" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="48"/>
-      <c r="B11" s="31" t="s">
+      <c r="A11" s="47"/>
+      <c r="B11" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="C11" s="32" t="s">
+      <c r="C11" s="33" t="s">
         <v>256</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E11" s="46" t="s">
-        <v>294</v>
-      </c>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="29"/>
-      <c r="K11" s="30"/>
-      <c r="L11" s="30"/>
-      <c r="M11" s="30"/>
-      <c r="N11" s="30"/>
-      <c r="O11" s="30"/>
-      <c r="P11" s="30"/>
-      <c r="Q11" s="30"/>
-      <c r="R11" s="30"/>
-      <c r="S11" s="30"/>
-      <c r="T11" s="30"/>
-      <c r="U11" s="30"/>
-      <c r="V11" s="30"/>
-      <c r="W11" s="30"/>
-      <c r="X11" s="30"/>
-      <c r="Y11" s="30"/>
-      <c r="Z11" s="30"/>
-      <c r="AA11" s="30"/>
-      <c r="AB11" s="30"/>
+      <c r="E11" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="31"/>
+      <c r="O11" s="31"/>
+      <c r="P11" s="31"/>
+      <c r="Q11" s="31"/>
+      <c r="R11" s="31"/>
+      <c r="S11" s="31"/>
+      <c r="T11" s="31"/>
+      <c r="U11" s="31"/>
+      <c r="V11" s="31"/>
+      <c r="W11" s="31"/>
+      <c r="X11" s="31"/>
+      <c r="Y11" s="31"/>
+      <c r="Z11" s="31"/>
+      <c r="AA11" s="31"/>
+      <c r="AB11" s="31"/>
     </row>
     <row r="12" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="48"/>
-      <c r="B12" s="31" t="s">
+      <c r="A12" s="47"/>
+      <c r="B12" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C12" s="32" t="s">
+      <c r="C12" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="D12" s="38" t="s">
+      <c r="D12" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E12" s="29" t="s">
+      <c r="E12" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="30"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-      <c r="P12" s="30"/>
-      <c r="Q12" s="30"/>
-      <c r="R12" s="30"/>
-      <c r="S12" s="30"/>
-      <c r="T12" s="30"/>
-      <c r="U12" s="30"/>
-      <c r="V12" s="30"/>
-      <c r="W12" s="30"/>
-      <c r="X12" s="30"/>
-      <c r="Y12" s="30"/>
-      <c r="Z12" s="30"/>
-      <c r="AA12" s="30"/>
-      <c r="AB12" s="30"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="31"/>
+      <c r="O12" s="31"/>
+      <c r="P12" s="31"/>
+      <c r="Q12" s="31"/>
+      <c r="R12" s="31"/>
+      <c r="S12" s="31"/>
+      <c r="T12" s="31"/>
+      <c r="U12" s="31"/>
+      <c r="V12" s="31"/>
+      <c r="W12" s="31"/>
+      <c r="X12" s="31"/>
+      <c r="Y12" s="31"/>
+      <c r="Z12" s="31"/>
+      <c r="AA12" s="31"/>
+      <c r="AB12" s="31"/>
     </row>
     <row r="13" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="47" t="s">
+      <c r="A13" s="46" t="s">
         <v>239</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="34" t="s">
         <v>254</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E13" s="29" t="s">
+      <c r="E13" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="29" t="s">
+      <c r="F13" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="29" t="s">
+      <c r="G13" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="H13" s="30"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
-      <c r="K13" s="30"/>
-      <c r="L13" s="30"/>
-      <c r="M13" s="30"/>
-      <c r="N13" s="30"/>
-      <c r="O13" s="30"/>
-      <c r="P13" s="30"/>
-      <c r="Q13" s="30"/>
-      <c r="R13" s="30"/>
-      <c r="S13" s="30"/>
-      <c r="T13" s="30"/>
-      <c r="U13" s="30"/>
-      <c r="V13" s="30"/>
-      <c r="W13" s="30"/>
-      <c r="X13" s="30"/>
-      <c r="Y13" s="30"/>
-      <c r="Z13" s="30"/>
-      <c r="AA13" s="30"/>
-      <c r="AB13" s="30"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
+      <c r="O13" s="31"/>
+      <c r="P13" s="31"/>
+      <c r="Q13" s="31"/>
+      <c r="R13" s="31"/>
+      <c r="S13" s="31"/>
+      <c r="T13" s="31"/>
+      <c r="U13" s="31"/>
+      <c r="V13" s="31"/>
+      <c r="W13" s="31"/>
+      <c r="X13" s="31"/>
+      <c r="Y13" s="31"/>
+      <c r="Z13" s="31"/>
+      <c r="AA13" s="31"/>
+      <c r="AB13" s="31"/>
     </row>
     <row r="14" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="47"/>
-      <c r="B14" s="31" t="s">
+      <c r="A14" s="46"/>
+      <c r="B14" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="C14" s="33" t="s">
+      <c r="C14" s="34" t="s">
         <v>254</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E14" s="29" t="s">
+      <c r="E14" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="30"/>
-      <c r="K14" s="30"/>
-      <c r="L14" s="30"/>
-      <c r="M14" s="30"/>
-      <c r="N14" s="30"/>
-      <c r="O14" s="30"/>
-      <c r="P14" s="30"/>
-      <c r="Q14" s="30"/>
-      <c r="R14" s="30"/>
-      <c r="S14" s="30"/>
-      <c r="T14" s="30"/>
-      <c r="U14" s="30"/>
-      <c r="V14" s="30"/>
-      <c r="W14" s="30"/>
-      <c r="X14" s="30"/>
-      <c r="Y14" s="30"/>
-      <c r="Z14" s="30"/>
-      <c r="AA14" s="30"/>
-      <c r="AB14" s="30"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="31"/>
+      <c r="O14" s="31"/>
+      <c r="P14" s="31"/>
+      <c r="Q14" s="31"/>
+      <c r="R14" s="31"/>
+      <c r="S14" s="31"/>
+      <c r="T14" s="31"/>
+      <c r="U14" s="31"/>
+      <c r="V14" s="31"/>
+      <c r="W14" s="31"/>
+      <c r="X14" s="31"/>
+      <c r="Y14" s="31"/>
+      <c r="Z14" s="31"/>
+      <c r="AA14" s="31"/>
+      <c r="AB14" s="31"/>
     </row>
     <row r="15" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="47"/>
-      <c r="B15" s="31" t="s">
+      <c r="A15" s="46"/>
+      <c r="B15" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="33" t="s">
         <v>258</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E15" s="29" t="s">
+      <c r="E15" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="F15" s="29" t="s">
+      <c r="F15" s="30" t="s">
         <v>143</v>
       </c>
-      <c r="G15" s="29" t="s">
+      <c r="G15" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="H15" s="29" t="s">
+      <c r="H15" s="30" t="s">
         <v>147</v>
       </c>
-      <c r="I15" s="29" t="s">
+      <c r="I15" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="J15" s="30"/>
-      <c r="K15" s="30"/>
-      <c r="L15" s="30"/>
-      <c r="M15" s="30"/>
-      <c r="N15" s="30"/>
-      <c r="O15" s="30"/>
-      <c r="P15" s="30"/>
-      <c r="Q15" s="30"/>
-      <c r="R15" s="30"/>
-      <c r="S15" s="30"/>
-      <c r="T15" s="30"/>
-      <c r="U15" s="30"/>
-      <c r="V15" s="30"/>
-      <c r="W15" s="30"/>
-      <c r="X15" s="30"/>
-      <c r="Y15" s="30"/>
-      <c r="Z15" s="30"/>
-      <c r="AA15" s="30"/>
-      <c r="AB15" s="30"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="31"/>
+      <c r="M15" s="31"/>
+      <c r="N15" s="31"/>
+      <c r="O15" s="31"/>
+      <c r="P15" s="31"/>
+      <c r="Q15" s="31"/>
+      <c r="R15" s="31"/>
+      <c r="S15" s="31"/>
+      <c r="T15" s="31"/>
+      <c r="U15" s="31"/>
+      <c r="V15" s="31"/>
+      <c r="W15" s="31"/>
+      <c r="X15" s="31"/>
+      <c r="Y15" s="31"/>
+      <c r="Z15" s="31"/>
+      <c r="AA15" s="31"/>
+      <c r="AB15" s="31"/>
     </row>
     <row r="16" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="34" t="s">
+      <c r="A16" s="35" t="s">
         <v>240</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="34" t="s">
         <v>259</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E16" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="F16" s="29" t="s">
+      <c r="F16" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="30"/>
-      <c r="K16" s="30"/>
-      <c r="L16" s="30"/>
-      <c r="M16" s="30"/>
-      <c r="N16" s="30"/>
-      <c r="O16" s="30"/>
-      <c r="P16" s="30"/>
-      <c r="Q16" s="30"/>
-      <c r="R16" s="30"/>
-      <c r="S16" s="30"/>
-      <c r="T16" s="30"/>
-      <c r="U16" s="30"/>
-      <c r="V16" s="30"/>
-      <c r="W16" s="30"/>
-      <c r="X16" s="30"/>
-      <c r="Y16" s="30"/>
-      <c r="Z16" s="30"/>
-      <c r="AA16" s="30"/>
-      <c r="AB16" s="30"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="31"/>
+      <c r="O16" s="31"/>
+      <c r="P16" s="31"/>
+      <c r="Q16" s="31"/>
+      <c r="R16" s="31"/>
+      <c r="S16" s="31"/>
+      <c r="T16" s="31"/>
+      <c r="U16" s="31"/>
+      <c r="V16" s="31"/>
+      <c r="W16" s="31"/>
+      <c r="X16" s="31"/>
+      <c r="Y16" s="31"/>
+      <c r="Z16" s="31"/>
+      <c r="AA16" s="31"/>
+      <c r="AB16" s="31"/>
     </row>
     <row r="17" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="47" t="s">
         <v>241</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E17" s="29" t="s">
+      <c r="E17" s="30" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="30"/>
-      <c r="K17" s="30"/>
-      <c r="L17" s="30"/>
-      <c r="M17" s="30"/>
-      <c r="N17" s="30"/>
-      <c r="O17" s="30"/>
-      <c r="P17" s="30"/>
-      <c r="Q17" s="30"/>
-      <c r="R17" s="30"/>
-      <c r="S17" s="30"/>
-      <c r="T17" s="30"/>
-      <c r="U17" s="30"/>
-      <c r="V17" s="30"/>
-      <c r="W17" s="30"/>
-      <c r="X17" s="30"/>
-      <c r="Y17" s="30"/>
-      <c r="Z17" s="30"/>
-      <c r="AA17" s="30"/>
-      <c r="AB17" s="30"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="31"/>
+      <c r="M17" s="31"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="31"/>
+      <c r="P17" s="31"/>
+      <c r="Q17" s="31"/>
+      <c r="R17" s="31"/>
+      <c r="S17" s="31"/>
+      <c r="T17" s="31"/>
+      <c r="U17" s="31"/>
+      <c r="V17" s="31"/>
+      <c r="W17" s="31"/>
+      <c r="X17" s="31"/>
+      <c r="Y17" s="31"/>
+      <c r="Z17" s="31"/>
+      <c r="AA17" s="31"/>
+      <c r="AB17" s="31"/>
     </row>
     <row r="18" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="48"/>
-      <c r="B18" s="31" t="s">
+      <c r="A18" s="47"/>
+      <c r="B18" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="C18" s="32" t="s">
+      <c r="C18" s="33" t="s">
         <v>260</v>
       </c>
-      <c r="D18" s="38" t="s">
+      <c r="D18" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E18" s="29" t="s">
+      <c r="E18" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="G18" s="29" t="s">
+      <c r="G18" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="H18" s="29" t="s">
+      <c r="H18" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="30"/>
-      <c r="N18" s="30"/>
-      <c r="O18" s="30"/>
-      <c r="P18" s="30"/>
-      <c r="Q18" s="30"/>
-      <c r="R18" s="30"/>
-      <c r="S18" s="30"/>
-      <c r="T18" s="30"/>
-      <c r="U18" s="30"/>
-      <c r="V18" s="30"/>
-      <c r="W18" s="30"/>
-      <c r="X18" s="30"/>
-      <c r="Y18" s="30"/>
-      <c r="Z18" s="30"/>
-      <c r="AA18" s="30"/>
-      <c r="AB18" s="30"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="31"/>
+      <c r="M18" s="31"/>
+      <c r="N18" s="31"/>
+      <c r="O18" s="31"/>
+      <c r="P18" s="31"/>
+      <c r="Q18" s="31"/>
+      <c r="R18" s="31"/>
+      <c r="S18" s="31"/>
+      <c r="T18" s="31"/>
+      <c r="U18" s="31"/>
+      <c r="V18" s="31"/>
+      <c r="W18" s="31"/>
+      <c r="X18" s="31"/>
+      <c r="Y18" s="31"/>
+      <c r="Z18" s="31"/>
+      <c r="AA18" s="31"/>
+      <c r="AB18" s="31"/>
     </row>
     <row r="19" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="48"/>
-      <c r="B19" s="31" t="s">
+      <c r="A19" s="47"/>
+      <c r="B19" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C19" s="32" t="s">
+      <c r="C19" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E19" s="29" t="s">
+      <c r="E19" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
-      <c r="K19" s="30"/>
-      <c r="L19" s="30"/>
-      <c r="M19" s="30"/>
-      <c r="N19" s="30"/>
-      <c r="O19" s="30"/>
-      <c r="P19" s="30"/>
-      <c r="Q19" s="30"/>
-      <c r="R19" s="30"/>
-      <c r="S19" s="30"/>
-      <c r="T19" s="30"/>
-      <c r="U19" s="30"/>
-      <c r="V19" s="30"/>
-      <c r="W19" s="30"/>
-      <c r="X19" s="30"/>
-      <c r="Y19" s="30"/>
-      <c r="Z19" s="30"/>
-      <c r="AA19" s="30"/>
-      <c r="AB19" s="30"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="31"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="31"/>
+      <c r="M19" s="31"/>
+      <c r="N19" s="31"/>
+      <c r="O19" s="31"/>
+      <c r="P19" s="31"/>
+      <c r="Q19" s="31"/>
+      <c r="R19" s="31"/>
+      <c r="S19" s="31"/>
+      <c r="T19" s="31"/>
+      <c r="U19" s="31"/>
+      <c r="V19" s="31"/>
+      <c r="W19" s="31"/>
+      <c r="X19" s="31"/>
+      <c r="Y19" s="31"/>
+      <c r="Z19" s="31"/>
+      <c r="AA19" s="31"/>
+      <c r="AB19" s="31"/>
     </row>
     <row r="20" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="48"/>
-      <c r="B20" s="31" t="s">
+      <c r="A20" s="47"/>
+      <c r="B20" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C20" s="32" t="s">
+      <c r="C20" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="D20" s="38" t="s">
+      <c r="D20" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E20" s="29" t="s">
+      <c r="E20" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="F20" s="29" t="s">
+      <c r="F20" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="G20" s="29" t="s">
+      <c r="G20" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="H20" s="29" t="s">
+      <c r="H20" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="I20" s="29" t="s">
+      <c r="I20" s="30" t="s">
         <v>126</v>
       </c>
-      <c r="J20" s="29" t="s">
+      <c r="J20" s="30" t="s">
         <v>128</v>
       </c>
-      <c r="K20" s="29" t="s">
+      <c r="K20" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="L20" s="29" t="s">
+      <c r="L20" s="30" t="s">
         <v>132</v>
       </c>
-      <c r="M20" s="30"/>
-      <c r="N20" s="30"/>
-      <c r="O20" s="30"/>
-      <c r="P20" s="30"/>
-      <c r="Q20" s="30"/>
-      <c r="R20" s="30"/>
-      <c r="S20" s="30"/>
-      <c r="T20" s="30"/>
-      <c r="U20" s="30"/>
-      <c r="V20" s="30"/>
-      <c r="W20" s="30"/>
-      <c r="X20" s="30"/>
-      <c r="Y20" s="30"/>
-      <c r="Z20" s="30"/>
-      <c r="AA20" s="30"/>
-      <c r="AB20" s="30"/>
+      <c r="M20" s="31"/>
+      <c r="N20" s="31"/>
+      <c r="O20" s="31"/>
+      <c r="P20" s="31"/>
+      <c r="Q20" s="31"/>
+      <c r="R20" s="31"/>
+      <c r="S20" s="31"/>
+      <c r="T20" s="31"/>
+      <c r="U20" s="31"/>
+      <c r="V20" s="31"/>
+      <c r="W20" s="31"/>
+      <c r="X20" s="31"/>
+      <c r="Y20" s="31"/>
+      <c r="Z20" s="31"/>
+      <c r="AA20" s="31"/>
+      <c r="AB20" s="31"/>
     </row>
     <row r="21" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="34" t="s">
+      <c r="A21" s="35" t="s">
         <v>242</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C21" s="33" t="s">
+      <c r="C21" s="34" t="s">
         <v>261</v>
       </c>
-      <c r="D21" s="38" t="s">
+      <c r="D21" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E21" s="29" t="s">
+      <c r="E21" s="30" t="s">
         <v>157</v>
       </c>
-      <c r="F21" s="29" t="s">
+      <c r="F21" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="G21" s="29" t="s">
+      <c r="G21" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="H21" s="29" t="s">
+      <c r="H21" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="I21" s="29" t="s">
+      <c r="I21" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="J21" s="29" t="s">
+      <c r="J21" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="K21" s="29" t="s">
+      <c r="K21" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="L21" s="30"/>
-      <c r="M21" s="30"/>
-      <c r="N21" s="30"/>
-      <c r="O21" s="30"/>
-      <c r="P21" s="30"/>
-      <c r="Q21" s="30"/>
-      <c r="R21" s="30"/>
-      <c r="S21" s="30"/>
-      <c r="T21" s="30"/>
-      <c r="U21" s="30"/>
-      <c r="V21" s="30"/>
-      <c r="W21" s="30"/>
-      <c r="X21" s="30"/>
-      <c r="Y21" s="30"/>
-      <c r="Z21" s="30"/>
-      <c r="AA21" s="30"/>
-      <c r="AB21" s="30"/>
+      <c r="L21" s="31"/>
+      <c r="M21" s="31"/>
+      <c r="N21" s="31"/>
+      <c r="O21" s="31"/>
+      <c r="P21" s="31"/>
+      <c r="Q21" s="31"/>
+      <c r="R21" s="31"/>
+      <c r="S21" s="31"/>
+      <c r="T21" s="31"/>
+      <c r="U21" s="31"/>
+      <c r="V21" s="31"/>
+      <c r="W21" s="31"/>
+      <c r="X21" s="31"/>
+      <c r="Y21" s="31"/>
+      <c r="Z21" s="31"/>
+      <c r="AA21" s="31"/>
+      <c r="AB21" s="31"/>
     </row>
     <row r="22" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="46" t="s">
         <v>243</v>
       </c>
-      <c r="B22" s="31" t="s">
+      <c r="B22" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="33" t="s">
         <v>258</v>
       </c>
-      <c r="D22" s="38" t="s">
+      <c r="D22" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E22" s="29" t="s">
+      <c r="E22" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="F22" s="29" t="s">
+      <c r="F22" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="G22" s="29" t="s">
+      <c r="G22" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H22" s="29" t="s">
+      <c r="H22" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="I22" s="29" t="s">
+      <c r="I22" s="30" t="s">
         <v>179</v>
       </c>
-      <c r="J22" s="29" t="s">
+      <c r="J22" s="30" t="s">
         <v>181</v>
       </c>
-      <c r="K22" s="29" t="s">
+      <c r="K22" s="30" t="s">
         <v>183</v>
       </c>
-      <c r="L22" s="29" t="s">
+      <c r="L22" s="30" t="s">
         <v>185</v>
       </c>
-      <c r="M22" s="29" t="s">
+      <c r="M22" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="N22" s="29" t="s">
+      <c r="N22" s="30" t="s">
         <v>189</v>
       </c>
-      <c r="O22" s="29" t="s">
+      <c r="O22" s="30" t="s">
         <v>191</v>
       </c>
-      <c r="P22" s="30"/>
-      <c r="Q22" s="30"/>
-      <c r="R22" s="30"/>
-      <c r="S22" s="30"/>
-      <c r="T22" s="30"/>
-      <c r="U22" s="30"/>
-      <c r="V22" s="30"/>
-      <c r="W22" s="30"/>
-      <c r="X22" s="30"/>
-      <c r="Y22" s="30"/>
-      <c r="Z22" s="30"/>
-      <c r="AA22" s="30"/>
-      <c r="AB22" s="30"/>
+      <c r="P22" s="31"/>
+      <c r="Q22" s="31"/>
+      <c r="R22" s="31"/>
+      <c r="S22" s="31"/>
+      <c r="T22" s="31"/>
+      <c r="U22" s="31"/>
+      <c r="V22" s="31"/>
+      <c r="W22" s="31"/>
+      <c r="X22" s="31"/>
+      <c r="Y22" s="31"/>
+      <c r="Z22" s="31"/>
+      <c r="AA22" s="31"/>
+      <c r="AB22" s="31"/>
     </row>
     <row r="23" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="47"/>
-      <c r="B23" s="31" t="s">
+      <c r="A23" s="46"/>
+      <c r="B23" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C23" s="32" t="s">
+      <c r="C23" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="D23" s="38" t="s">
+      <c r="D23" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E23" s="29" t="s">
+      <c r="E23" s="30" t="s">
         <v>134</v>
       </c>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="30"/>
-      <c r="K23" s="30"/>
-      <c r="L23" s="30"/>
-      <c r="M23" s="30"/>
-      <c r="N23" s="30"/>
-      <c r="O23" s="30"/>
-      <c r="P23" s="30"/>
-      <c r="Q23" s="30"/>
-      <c r="R23" s="30"/>
-      <c r="S23" s="30"/>
-      <c r="T23" s="30"/>
-      <c r="U23" s="30"/>
-      <c r="V23" s="30"/>
-      <c r="W23" s="30"/>
-      <c r="X23" s="30"/>
-      <c r="Y23" s="30"/>
-      <c r="Z23" s="30"/>
-      <c r="AA23" s="30"/>
-      <c r="AB23" s="30"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
+      <c r="L23" s="31"/>
+      <c r="M23" s="31"/>
+      <c r="N23" s="31"/>
+      <c r="O23" s="31"/>
+      <c r="P23" s="31"/>
+      <c r="Q23" s="31"/>
+      <c r="R23" s="31"/>
+      <c r="S23" s="31"/>
+      <c r="T23" s="31"/>
+      <c r="U23" s="31"/>
+      <c r="V23" s="31"/>
+      <c r="W23" s="31"/>
+      <c r="X23" s="31"/>
+      <c r="Y23" s="31"/>
+      <c r="Z23" s="31"/>
+      <c r="AA23" s="31"/>
+      <c r="AB23" s="31"/>
     </row>
     <row r="24" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="34" t="s">
+      <c r="A24" s="35" t="s">
         <v>244</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="C24" s="32" t="s">
+      <c r="C24" s="33" t="s">
         <v>262</v>
       </c>
-      <c r="D24" s="38" t="s">
+      <c r="D24" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="30"/>
-      <c r="K24" s="30"/>
-      <c r="L24" s="30"/>
-      <c r="M24" s="30"/>
-      <c r="N24" s="30"/>
-      <c r="O24" s="30"/>
-      <c r="P24" s="30"/>
-      <c r="Q24" s="30"/>
-      <c r="R24" s="30"/>
-      <c r="S24" s="30"/>
-      <c r="T24" s="30"/>
-      <c r="U24" s="30"/>
-      <c r="V24" s="30"/>
-      <c r="W24" s="30"/>
-      <c r="X24" s="30"/>
-      <c r="Y24" s="30"/>
-      <c r="Z24" s="30"/>
-      <c r="AA24" s="30"/>
-      <c r="AB24" s="30"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="31"/>
+      <c r="M24" s="31"/>
+      <c r="N24" s="31"/>
+      <c r="O24" s="31"/>
+      <c r="P24" s="31"/>
+      <c r="Q24" s="31"/>
+      <c r="R24" s="31"/>
+      <c r="S24" s="31"/>
+      <c r="T24" s="31"/>
+      <c r="U24" s="31"/>
+      <c r="V24" s="31"/>
+      <c r="W24" s="31"/>
+      <c r="X24" s="31"/>
+      <c r="Y24" s="31"/>
+      <c r="Z24" s="31"/>
+      <c r="AA24" s="31"/>
+      <c r="AB24" s="31"/>
     </row>
     <row r="25" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="47" t="s">
+      <c r="A25" s="46" t="s">
         <v>246</v>
       </c>
-      <c r="B25" s="43" t="s">
+      <c r="B25" s="45" t="s">
         <v>233</v>
       </c>
-      <c r="C25" s="32" t="s">
+      <c r="C25" s="33" t="s">
         <v>256</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="D25" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E25" s="29" t="s">
+      <c r="E25" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="F25" s="29" t="s">
+      <c r="F25" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="29" t="s">
+      <c r="G25" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="H25" s="29" t="s">
+      <c r="H25" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="I25" s="30"/>
-      <c r="J25" s="30"/>
-      <c r="K25" s="30"/>
-      <c r="L25" s="30"/>
-      <c r="M25" s="30"/>
-      <c r="N25" s="30"/>
-      <c r="O25" s="30"/>
-      <c r="P25" s="30"/>
-      <c r="Q25" s="30"/>
-      <c r="R25" s="30"/>
-      <c r="S25" s="30"/>
-      <c r="T25" s="30"/>
-      <c r="U25" s="30"/>
-      <c r="V25" s="30"/>
-      <c r="W25" s="30"/>
-      <c r="X25" s="30"/>
-      <c r="Y25" s="30"/>
-      <c r="Z25" s="30"/>
-      <c r="AA25" s="30"/>
-      <c r="AB25" s="30"/>
+      <c r="I25" s="31"/>
+      <c r="J25" s="31"/>
+      <c r="K25" s="31"/>
+      <c r="L25" s="31"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="31"/>
+      <c r="O25" s="31"/>
+      <c r="P25" s="31"/>
+      <c r="Q25" s="31"/>
+      <c r="R25" s="31"/>
+      <c r="S25" s="31"/>
+      <c r="T25" s="31"/>
+      <c r="U25" s="31"/>
+      <c r="V25" s="31"/>
+      <c r="W25" s="31"/>
+      <c r="X25" s="31"/>
+      <c r="Y25" s="31"/>
+      <c r="Z25" s="31"/>
+      <c r="AA25" s="31"/>
+      <c r="AB25" s="31"/>
     </row>
     <row r="26" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="47"/>
-      <c r="B26" s="43" t="s">
+      <c r="A26" s="46"/>
+      <c r="B26" s="45" t="s">
         <v>232</v>
       </c>
-      <c r="C26" s="32" t="s">
+      <c r="C26" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D26" s="38" t="s">
+      <c r="D26" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E26" s="29" t="s">
+      <c r="E26" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="F26" s="29" t="s">
+      <c r="F26" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="29" t="s">
+      <c r="G26" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="H26" s="29" t="s">
+      <c r="H26" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="I26" s="29" t="s">
+      <c r="I26" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="J26" s="29" t="s">
+      <c r="J26" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="K26" s="30"/>
-      <c r="L26" s="30"/>
-      <c r="M26" s="30"/>
-      <c r="N26" s="30"/>
-      <c r="O26" s="30"/>
-      <c r="P26" s="30"/>
-      <c r="Q26" s="30"/>
-      <c r="R26" s="30"/>
-      <c r="S26" s="30"/>
-      <c r="T26" s="30"/>
-      <c r="U26" s="30"/>
-      <c r="V26" s="30"/>
-      <c r="W26" s="30"/>
-      <c r="X26" s="30"/>
-      <c r="Y26" s="30"/>
-      <c r="Z26" s="30"/>
-      <c r="AA26" s="30"/>
-      <c r="AB26" s="30"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="31"/>
+      <c r="M26" s="31"/>
+      <c r="N26" s="31"/>
+      <c r="O26" s="31"/>
+      <c r="P26" s="31"/>
+      <c r="Q26" s="31"/>
+      <c r="R26" s="31"/>
+      <c r="S26" s="31"/>
+      <c r="T26" s="31"/>
+      <c r="U26" s="31"/>
+      <c r="V26" s="31"/>
+      <c r="W26" s="31"/>
+      <c r="X26" s="31"/>
+      <c r="Y26" s="31"/>
+      <c r="Z26" s="31"/>
+      <c r="AA26" s="31"/>
+      <c r="AB26" s="31"/>
     </row>
     <row r="27" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="47"/>
-      <c r="B27" s="31" t="s">
+      <c r="A27" s="46"/>
+      <c r="B27" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C27" s="32" t="s">
+      <c r="C27" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="D27" s="38" t="s">
+      <c r="D27" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="29"/>
-      <c r="K27" s="30"/>
-      <c r="L27" s="30"/>
-      <c r="M27" s="30"/>
-      <c r="N27" s="30"/>
-      <c r="O27" s="30"/>
-      <c r="P27" s="30"/>
-      <c r="Q27" s="30"/>
-      <c r="R27" s="30"/>
-      <c r="S27" s="30"/>
-      <c r="T27" s="30"/>
-      <c r="U27" s="30"/>
-      <c r="V27" s="30"/>
-      <c r="W27" s="30"/>
-      <c r="X27" s="30"/>
-      <c r="Y27" s="30"/>
-      <c r="Z27" s="30"/>
-      <c r="AA27" s="30"/>
-      <c r="AB27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="30"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="31"/>
+      <c r="M27" s="31"/>
+      <c r="N27" s="31"/>
+      <c r="O27" s="31"/>
+      <c r="P27" s="31"/>
+      <c r="Q27" s="31"/>
+      <c r="R27" s="31"/>
+      <c r="S27" s="31"/>
+      <c r="T27" s="31"/>
+      <c r="U27" s="31"/>
+      <c r="V27" s="31"/>
+      <c r="W27" s="31"/>
+      <c r="X27" s="31"/>
+      <c r="Y27" s="31"/>
+      <c r="Z27" s="31"/>
+      <c r="AA27" s="31"/>
+      <c r="AB27" s="31"/>
     </row>
     <row r="28" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="47"/>
-      <c r="B28" s="31" t="s">
+      <c r="A28" s="46"/>
+      <c r="B28" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C28" s="32" t="s">
+      <c r="C28" s="33" t="s">
         <v>258</v>
       </c>
-      <c r="D28" s="38" t="s">
+      <c r="D28" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E28" s="29" t="s">
+      <c r="E28" s="30" t="s">
         <v>136</v>
       </c>
-      <c r="F28" s="29" t="s">
+      <c r="F28" s="30" t="s">
         <v>139</v>
       </c>
-      <c r="G28" s="29" t="s">
+      <c r="G28" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="H28" s="29" t="s">
+      <c r="H28" s="30" t="s">
         <v>143</v>
       </c>
-      <c r="I28" s="30"/>
-      <c r="J28" s="30"/>
-      <c r="K28" s="30"/>
-      <c r="L28" s="30"/>
-      <c r="M28" s="30"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="30"/>
-      <c r="P28" s="30"/>
-      <c r="Q28" s="30"/>
-      <c r="R28" s="30"/>
-      <c r="S28" s="30"/>
-      <c r="T28" s="30"/>
-      <c r="U28" s="30"/>
-      <c r="V28" s="30"/>
-      <c r="W28" s="30"/>
-      <c r="X28" s="30"/>
-      <c r="Y28" s="30"/>
-      <c r="Z28" s="30"/>
-      <c r="AA28" s="30"/>
-      <c r="AB28" s="30"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="31"/>
+      <c r="M28" s="31"/>
+      <c r="N28" s="31"/>
+      <c r="O28" s="31"/>
+      <c r="P28" s="31"/>
+      <c r="Q28" s="31"/>
+      <c r="R28" s="31"/>
+      <c r="S28" s="31"/>
+      <c r="T28" s="31"/>
+      <c r="U28" s="31"/>
+      <c r="V28" s="31"/>
+      <c r="W28" s="31"/>
+      <c r="X28" s="31"/>
+      <c r="Y28" s="31"/>
+      <c r="Z28" s="31"/>
+      <c r="AA28" s="31"/>
+      <c r="AB28" s="31"/>
     </row>
     <row r="29" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="34" t="s">
+      <c r="A29" s="35" t="s">
         <v>247</v>
       </c>
-      <c r="B29" s="31" t="s">
+      <c r="B29" s="32" t="s">
         <v>282</v>
       </c>
-      <c r="C29" s="32" t="s">
+      <c r="C29" s="33" t="s">
         <v>263</v>
       </c>
-      <c r="D29" s="38" t="s">
+      <c r="D29" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="30"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30"/>
-      <c r="O29" s="30"/>
-      <c r="P29" s="30"/>
-      <c r="Q29" s="30"/>
-      <c r="R29" s="30"/>
-      <c r="S29" s="30"/>
-      <c r="T29" s="30"/>
-      <c r="U29" s="30"/>
-      <c r="V29" s="30"/>
-      <c r="W29" s="30"/>
-      <c r="X29" s="30"/>
-      <c r="Y29" s="30"/>
-      <c r="Z29" s="30"/>
-      <c r="AA29" s="30"/>
-      <c r="AB29" s="30"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="31"/>
+      <c r="K29" s="31"/>
+      <c r="L29" s="31"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="31"/>
+      <c r="O29" s="31"/>
+      <c r="P29" s="31"/>
+      <c r="Q29" s="31"/>
+      <c r="R29" s="31"/>
+      <c r="S29" s="31"/>
+      <c r="T29" s="31"/>
+      <c r="U29" s="31"/>
+      <c r="V29" s="31"/>
+      <c r="W29" s="31"/>
+      <c r="X29" s="31"/>
+      <c r="Y29" s="31"/>
+      <c r="Z29" s="31"/>
+      <c r="AA29" s="31"/>
+      <c r="AB29" s="31"/>
     </row>
     <row r="30" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="34" t="s">
+      <c r="A30" s="35" t="s">
         <v>248</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="32" t="s">
         <v>283</v>
       </c>
-      <c r="C30" s="32" t="s">
+      <c r="C30" s="33" t="s">
         <v>264</v>
       </c>
-      <c r="D30" s="38" t="s">
+      <c r="D30" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E30" s="30"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
-      <c r="K30" s="30"/>
-      <c r="L30" s="30"/>
-      <c r="M30" s="30"/>
-      <c r="N30" s="30"/>
-      <c r="O30" s="30"/>
-      <c r="P30" s="30"/>
-      <c r="Q30" s="30"/>
-      <c r="R30" s="30"/>
-      <c r="S30" s="30"/>
-      <c r="T30" s="30"/>
-      <c r="U30" s="30"/>
-      <c r="V30" s="30"/>
-      <c r="W30" s="30"/>
-      <c r="X30" s="30"/>
-      <c r="Y30" s="30"/>
-      <c r="Z30" s="30"/>
-      <c r="AA30" s="30"/>
-      <c r="AB30" s="30"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="31"/>
+      <c r="J30" s="31"/>
+      <c r="K30" s="31"/>
+      <c r="L30" s="31"/>
+      <c r="M30" s="31"/>
+      <c r="N30" s="31"/>
+      <c r="O30" s="31"/>
+      <c r="P30" s="31"/>
+      <c r="Q30" s="31"/>
+      <c r="R30" s="31"/>
+      <c r="S30" s="31"/>
+      <c r="T30" s="31"/>
+      <c r="U30" s="31"/>
+      <c r="V30" s="31"/>
+      <c r="W30" s="31"/>
+      <c r="X30" s="31"/>
+      <c r="Y30" s="31"/>
+      <c r="Z30" s="31"/>
+      <c r="AA30" s="31"/>
+      <c r="AB30" s="31"/>
     </row>
     <row r="31" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="34" t="s">
+      <c r="A31" s="35" t="s">
         <v>249</v>
       </c>
-      <c r="B31" s="35" t="s">
+      <c r="B31" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="C31" s="32" t="s">
+      <c r="C31" s="33" t="s">
         <v>262</v>
       </c>
-      <c r="D31" s="38" t="s">
+      <c r="D31" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="30"/>
-      <c r="J31" s="30"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="30"/>
-      <c r="N31" s="30"/>
-      <c r="O31" s="30"/>
-      <c r="P31" s="30"/>
-      <c r="Q31" s="30"/>
-      <c r="R31" s="30"/>
-      <c r="S31" s="30"/>
-      <c r="T31" s="30"/>
-      <c r="U31" s="30"/>
-      <c r="V31" s="30"/>
-      <c r="W31" s="30"/>
-      <c r="X31" s="30"/>
-      <c r="Y31" s="30"/>
-      <c r="Z31" s="30"/>
-      <c r="AA31" s="30"/>
-      <c r="AB31" s="30"/>
+      <c r="E31" s="31"/>
+      <c r="F31" s="31"/>
+      <c r="G31" s="31"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="31"/>
+      <c r="J31" s="31"/>
+      <c r="K31" s="31"/>
+      <c r="L31" s="31"/>
+      <c r="M31" s="31"/>
+      <c r="N31" s="31"/>
+      <c r="O31" s="31"/>
+      <c r="P31" s="31"/>
+      <c r="Q31" s="31"/>
+      <c r="R31" s="31"/>
+      <c r="S31" s="31"/>
+      <c r="T31" s="31"/>
+      <c r="U31" s="31"/>
+      <c r="V31" s="31"/>
+      <c r="W31" s="31"/>
+      <c r="X31" s="31"/>
+      <c r="Y31" s="31"/>
+      <c r="Z31" s="31"/>
+      <c r="AA31" s="31"/>
+      <c r="AB31" s="31"/>
     </row>
     <row r="32" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="46" t="s">
         <v>250</v>
       </c>
-      <c r="B32" s="43" t="s">
+      <c r="B32" s="45" t="s">
         <v>233</v>
       </c>
-      <c r="C32" s="32" t="s">
+      <c r="C32" s="33" t="s">
         <v>256</v>
       </c>
-      <c r="D32" s="38" t="s">
+      <c r="D32" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E32" s="29" t="s">
+      <c r="E32" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="29" t="s">
+      <c r="F32" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="G32" s="29" t="s">
+      <c r="G32" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="H32" s="29" t="s">
+      <c r="H32" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="I32" s="29" t="s">
+      <c r="I32" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="J32" s="29" t="s">
+      <c r="J32" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="K32" s="29" t="s">
+      <c r="K32" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="L32" s="29" t="s">
+      <c r="L32" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="M32" s="29" t="s">
+      <c r="M32" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="N32" s="29" t="s">
+      <c r="N32" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="O32" s="29" t="s">
+      <c r="O32" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="P32" s="30"/>
-      <c r="Q32" s="30"/>
-      <c r="R32" s="30"/>
-      <c r="S32" s="30"/>
-      <c r="T32" s="30"/>
-      <c r="U32" s="30"/>
-      <c r="V32" s="30"/>
-      <c r="W32" s="30"/>
-      <c r="X32" s="30"/>
-      <c r="Y32" s="30"/>
-      <c r="Z32" s="30"/>
-      <c r="AA32" s="30"/>
-      <c r="AB32" s="30"/>
+      <c r="P32" s="31"/>
+      <c r="Q32" s="31"/>
+      <c r="R32" s="31"/>
+      <c r="S32" s="31"/>
+      <c r="T32" s="31"/>
+      <c r="U32" s="31"/>
+      <c r="V32" s="31"/>
+      <c r="W32" s="31"/>
+      <c r="X32" s="31"/>
+      <c r="Y32" s="31"/>
+      <c r="Z32" s="31"/>
+      <c r="AA32" s="31"/>
+      <c r="AB32" s="31"/>
     </row>
     <row r="33" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="47"/>
-      <c r="B33" s="43" t="s">
+      <c r="A33" s="46"/>
+      <c r="B33" s="45" t="s">
         <v>232</v>
       </c>
-      <c r="C33" s="32" t="s">
+      <c r="C33" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D33" s="38" t="s">
+      <c r="D33" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E33" s="29" t="s">
+      <c r="E33" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="F33" s="29" t="s">
+      <c r="F33" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="30"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="30"/>
-      <c r="M33" s="30"/>
-      <c r="N33" s="30"/>
-      <c r="O33" s="30"/>
-      <c r="P33" s="30"/>
-      <c r="Q33" s="30"/>
-      <c r="R33" s="30"/>
-      <c r="S33" s="30"/>
-      <c r="T33" s="30"/>
-      <c r="U33" s="30"/>
-      <c r="V33" s="30"/>
-      <c r="W33" s="30"/>
-      <c r="X33" s="30"/>
-      <c r="Y33" s="30"/>
-      <c r="Z33" s="30"/>
-      <c r="AA33" s="30"/>
-      <c r="AB33" s="30"/>
+      <c r="G33" s="31"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="31"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="31"/>
+      <c r="O33" s="31"/>
+      <c r="P33" s="31"/>
+      <c r="Q33" s="31"/>
+      <c r="R33" s="31"/>
+      <c r="S33" s="31"/>
+      <c r="T33" s="31"/>
+      <c r="U33" s="31"/>
+      <c r="V33" s="31"/>
+      <c r="W33" s="31"/>
+      <c r="X33" s="31"/>
+      <c r="Y33" s="31"/>
+      <c r="Z33" s="31"/>
+      <c r="AA33" s="31"/>
+      <c r="AB33" s="31"/>
     </row>
     <row r="34" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="47"/>
-      <c r="B34" s="31" t="s">
+      <c r="A34" s="46"/>
+      <c r="B34" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C34" s="32" t="s">
+      <c r="C34" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="D34" s="38" t="s">
+      <c r="D34" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E34" s="42" t="s">
+      <c r="E34" s="44" t="s">
         <v>114</v>
       </c>
-      <c r="F34" s="42" t="s">
+      <c r="F34" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="G34" s="42" t="s">
+      <c r="G34" s="44" t="s">
         <v>120</v>
       </c>
-      <c r="H34" s="42" t="s">
+      <c r="H34" s="44" t="s">
         <v>122</v>
       </c>
-      <c r="I34" s="42" t="s">
+      <c r="I34" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="J34" s="42" t="s">
+      <c r="J34" s="44" t="s">
         <v>126</v>
       </c>
-      <c r="K34" s="42" t="s">
+      <c r="K34" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="L34" s="42" t="s">
+      <c r="L34" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="M34" s="42" t="s">
+      <c r="M34" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="N34" s="42" t="s">
+      <c r="N34" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="O34" s="30"/>
-      <c r="P34" s="30"/>
-      <c r="Q34" s="30"/>
-      <c r="R34" s="30"/>
-      <c r="S34" s="30"/>
-      <c r="T34" s="30"/>
-      <c r="U34" s="30"/>
-      <c r="V34" s="30"/>
-      <c r="W34" s="30"/>
-      <c r="X34" s="30"/>
-      <c r="Y34" s="30"/>
-      <c r="Z34" s="30"/>
-      <c r="AA34" s="30"/>
-      <c r="AB34" s="30"/>
+      <c r="O34" s="31"/>
+      <c r="P34" s="31"/>
+      <c r="Q34" s="31"/>
+      <c r="R34" s="31"/>
+      <c r="S34" s="31"/>
+      <c r="T34" s="31"/>
+      <c r="U34" s="31"/>
+      <c r="V34" s="31"/>
+      <c r="W34" s="31"/>
+      <c r="X34" s="31"/>
+      <c r="Y34" s="31"/>
+      <c r="Z34" s="31"/>
+      <c r="AA34" s="31"/>
+      <c r="AB34" s="31"/>
     </row>
     <row r="35" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="47"/>
-      <c r="B35" s="31" t="s">
+      <c r="A35" s="46"/>
+      <c r="B35" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="C35" s="32" t="s">
+      <c r="C35" s="33" t="s">
         <v>258</v>
       </c>
-      <c r="D35" s="38" t="s">
+      <c r="D35" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E35" s="29" t="s">
+      <c r="E35" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="F35" s="29" t="s">
+      <c r="F35" s="30" t="s">
         <v>147</v>
       </c>
-      <c r="G35" s="29" t="s">
+      <c r="G35" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="H35" s="29" t="s">
+      <c r="H35" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="I35" s="29" t="s">
+      <c r="I35" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="J35" s="29" t="s">
+      <c r="J35" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="K35" s="29" t="s">
+      <c r="K35" s="30" t="s">
         <v>157</v>
       </c>
-      <c r="L35" s="29" t="s">
+      <c r="L35" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="M35" s="29" t="s">
+      <c r="M35" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="N35" s="29" t="s">
+      <c r="N35" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="O35" s="29" t="s">
+      <c r="O35" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="P35" s="29" t="s">
+      <c r="P35" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="Q35" s="29" t="s">
+      <c r="Q35" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="R35" s="29" t="s">
+      <c r="R35" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="S35" s="29" t="s">
+      <c r="S35" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="T35" s="29" t="s">
+      <c r="T35" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="U35" s="29" t="s">
+      <c r="U35" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="V35" s="29" t="s">
+      <c r="V35" s="30" t="s">
         <v>179</v>
       </c>
-      <c r="W35" s="29" t="s">
+      <c r="W35" s="30" t="s">
         <v>181</v>
       </c>
-      <c r="X35" s="29" t="s">
+      <c r="X35" s="30" t="s">
         <v>183</v>
       </c>
-      <c r="Y35" s="29" t="s">
+      <c r="Y35" s="30" t="s">
         <v>185</v>
       </c>
-      <c r="Z35" s="29" t="s">
+      <c r="Z35" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="AA35" s="29" t="s">
+      <c r="AA35" s="30" t="s">
         <v>189</v>
       </c>
-      <c r="AB35" s="29" t="s">
+      <c r="AB35" s="30" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="36" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="34" t="s">
+      <c r="A36" s="35" t="s">
         <v>251</v>
       </c>
-      <c r="B36" s="31" t="s">
+      <c r="B36" s="32" t="s">
         <v>282</v>
       </c>
-      <c r="C36" s="32" t="s">
+      <c r="C36" s="33" t="s">
         <v>263</v>
       </c>
-      <c r="D36" s="38" t="s">
+      <c r="D36" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E36" s="30"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="30"/>
-      <c r="J36" s="30"/>
-      <c r="K36" s="30"/>
-      <c r="L36" s="30"/>
-      <c r="M36" s="30"/>
-      <c r="N36" s="30"/>
-      <c r="O36" s="30"/>
-      <c r="P36" s="30"/>
-      <c r="Q36" s="30"/>
-      <c r="R36" s="30"/>
-      <c r="S36" s="30"/>
-      <c r="T36" s="30"/>
-      <c r="U36" s="30"/>
-      <c r="V36" s="30"/>
-      <c r="W36" s="30"/>
-      <c r="X36" s="30"/>
-      <c r="Y36" s="30"/>
-      <c r="Z36" s="30"/>
-      <c r="AA36" s="30"/>
-      <c r="AB36" s="30"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="31"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="31"/>
+      <c r="J36" s="31"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="31"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="31"/>
+      <c r="O36" s="31"/>
+      <c r="P36" s="31"/>
+      <c r="Q36" s="31"/>
+      <c r="R36" s="31"/>
+      <c r="S36" s="31"/>
+      <c r="T36" s="31"/>
+      <c r="U36" s="31"/>
+      <c r="V36" s="31"/>
+      <c r="W36" s="31"/>
+      <c r="X36" s="31"/>
+      <c r="Y36" s="31"/>
+      <c r="Z36" s="31"/>
+      <c r="AA36" s="31"/>
+      <c r="AB36" s="31"/>
     </row>
     <row r="37" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="36" t="s">
+      <c r="A37" s="37" t="s">
         <v>252</v>
       </c>
-      <c r="B37" s="31" t="s">
+      <c r="B37" s="32" t="s">
         <v>283</v>
       </c>
-      <c r="C37" s="32" t="s">
+      <c r="C37" s="33" t="s">
         <v>264</v>
       </c>
-      <c r="D37" s="38" t="s">
+      <c r="D37" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E37" s="30"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="30"/>
-      <c r="I37" s="30"/>
-      <c r="J37" s="30"/>
-      <c r="K37" s="30"/>
-      <c r="L37" s="30"/>
-      <c r="M37" s="30"/>
-      <c r="N37" s="30"/>
-      <c r="O37" s="30"/>
-      <c r="P37" s="30"/>
-      <c r="Q37" s="30"/>
-      <c r="R37" s="30"/>
-      <c r="S37" s="30"/>
-      <c r="T37" s="30"/>
-      <c r="U37" s="30"/>
-      <c r="V37" s="30"/>
-      <c r="W37" s="30"/>
-      <c r="X37" s="30"/>
-      <c r="Y37" s="30"/>
-      <c r="Z37" s="30"/>
-      <c r="AA37" s="30"/>
-      <c r="AB37" s="30"/>
+      <c r="E37" s="31"/>
+      <c r="F37" s="31"/>
+      <c r="G37" s="31"/>
+      <c r="H37" s="31"/>
+      <c r="I37" s="31"/>
+      <c r="J37" s="31"/>
+      <c r="K37" s="31"/>
+      <c r="L37" s="31"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="31"/>
+      <c r="O37" s="31"/>
+      <c r="P37" s="31"/>
+      <c r="Q37" s="31"/>
+      <c r="R37" s="31"/>
+      <c r="S37" s="31"/>
+      <c r="T37" s="31"/>
+      <c r="U37" s="31"/>
+      <c r="V37" s="31"/>
+      <c r="W37" s="31"/>
+      <c r="X37" s="31"/>
+      <c r="Y37" s="31"/>
+      <c r="Z37" s="31"/>
+      <c r="AA37" s="31"/>
+      <c r="AB37" s="31"/>
     </row>
     <row r="38" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="34" t="s">
+      <c r="A38" s="35" t="s">
         <v>253</v>
       </c>
-      <c r="B38" s="35" t="s">
+      <c r="B38" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="C38" s="32" t="s">
+      <c r="C38" s="33" t="s">
         <v>262</v>
       </c>
-      <c r="D38" s="38" t="s">
+      <c r="D38" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="E38" s="30"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30"/>
-      <c r="I38" s="30"/>
-      <c r="J38" s="30"/>
-      <c r="K38" s="30"/>
-      <c r="L38" s="30"/>
-      <c r="M38" s="30"/>
-      <c r="N38" s="30"/>
-      <c r="O38" s="30"/>
-      <c r="P38" s="30"/>
-      <c r="Q38" s="30"/>
-      <c r="R38" s="30"/>
-      <c r="S38" s="30"/>
-      <c r="T38" s="30"/>
-      <c r="U38" s="30"/>
-      <c r="V38" s="30"/>
-      <c r="W38" s="30"/>
-      <c r="X38" s="30"/>
-      <c r="Y38" s="30"/>
-      <c r="Z38" s="30"/>
-      <c r="AA38" s="30"/>
-      <c r="AB38" s="30"/>
+      <c r="E38" s="31"/>
+      <c r="F38" s="31"/>
+      <c r="G38" s="31"/>
+      <c r="H38" s="31"/>
+      <c r="I38" s="31"/>
+      <c r="J38" s="31"/>
+      <c r="K38" s="31"/>
+      <c r="L38" s="31"/>
+      <c r="M38" s="31"/>
+      <c r="N38" s="31"/>
+      <c r="O38" s="31"/>
+      <c r="P38" s="31"/>
+      <c r="Q38" s="31"/>
+      <c r="R38" s="31"/>
+      <c r="S38" s="31"/>
+      <c r="T38" s="31"/>
+      <c r="U38" s="31"/>
+      <c r="V38" s="31"/>
+      <c r="W38" s="31"/>
+      <c r="X38" s="31"/>
+      <c r="Y38" s="31"/>
+      <c r="Z38" s="31"/>
+      <c r="AA38" s="31"/>
+      <c r="AB38" s="31"/>
     </row>
     <row r="39" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C39" s="26"/>
     </row>
+    <row r="40" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C40" s="28"/>
+    </row>
     <row r="41" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C41" s="27"/>
     </row>
     <row r="42" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="C42" s="28"/>
+      <c r="C42" s="29"/>
     </row>
     <row r="43" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C43" s="26"/>
     </row>
+    <row r="44" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C44" s="28"/>
+    </row>
     <row r="45" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C45" s="27"/>
     </row>
     <row r="46" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C46" s="26"/>
     </row>
+    <row r="47" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C47" s="28"/>
+    </row>
+    <row r="48" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C48" s="28"/>
+    </row>
+    <row r="49" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C49" s="28"/>
+    </row>
+    <row r="50" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C50" s="28"/>
+    </row>
+    <row r="51" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C51" s="28"/>
+    </row>
+    <row r="52" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C52" s="28"/>
+    </row>
+    <row r="53" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C53" s="28"/>
+    </row>
+    <row r="54" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C54" s="28"/>
+    </row>
+    <row r="55" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C55" s="28"/>
+    </row>
+    <row r="56" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C56" s="28"/>
+    </row>
+    <row r="57" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C57" s="28"/>
+    </row>
+    <row r="58" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C58" s="28"/>
+    </row>
+    <row r="59" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C59" s="28"/>
+    </row>
+    <row r="60" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C60" s="28"/>
+    </row>
     <row r="61" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C61" s="27"/>
+    </row>
+    <row r="62" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C62" s="28"/>
+    </row>
+    <row r="63" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C63" s="28"/>
+    </row>
+    <row r="64" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C64" s="28"/>
+    </row>
+    <row r="65" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C65" s="28"/>
+    </row>
+    <row r="66" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C66" s="28"/>
+    </row>
+    <row r="67" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C67" s="28"/>
+    </row>
+    <row r="68" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C68" s="28"/>
+    </row>
+    <row r="69" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C69" s="28"/>
+    </row>
+    <row r="70" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C70" s="28"/>
+    </row>
+    <row r="71" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C71" s="28"/>
+    </row>
+    <row r="72" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C72" s="28"/>
+    </row>
+    <row r="73" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C73" s="28"/>
+    </row>
+    <row r="74" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C74" s="28"/>
+    </row>
+    <row r="75" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C75" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5980,703 +5913,703 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="2" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="42" t="s">
         <v>271</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="40"/>
-      <c r="M2" s="40"/>
-      <c r="N2" s="40"/>
-      <c r="O2" s="40"/>
-      <c r="P2" s="40"/>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="40"/>
-      <c r="S2" s="40"/>
-      <c r="T2" s="40"/>
-      <c r="U2" s="40"/>
-      <c r="V2" s="40"/>
-      <c r="W2" s="40"/>
-      <c r="X2" s="40"/>
-      <c r="Y2" s="40"/>
-      <c r="Z2" s="40"/>
-      <c r="AA2" s="40"/>
-      <c r="AB2" s="40"/>
-      <c r="AC2" s="40"/>
-      <c r="AD2" s="40"/>
-      <c r="AE2" s="40"/>
-      <c r="AF2" s="40"/>
-      <c r="AG2" s="40"/>
-      <c r="AH2" s="40"/>
-      <c r="AI2" s="40"/>
-      <c r="AJ2" s="40"/>
-      <c r="AK2" s="40"/>
-      <c r="AL2" s="40"/>
-      <c r="AM2" s="40"/>
-      <c r="AN2" s="40"/>
-      <c r="AO2" s="40"/>
-      <c r="AP2" s="40"/>
-      <c r="AQ2" s="40"/>
-      <c r="AR2" s="40"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="41"/>
+      <c r="R2" s="41"/>
+      <c r="S2" s="41"/>
+      <c r="T2" s="41"/>
+      <c r="U2" s="41"/>
+      <c r="V2" s="41"/>
+      <c r="W2" s="41"/>
+      <c r="X2" s="41"/>
+      <c r="Y2" s="41"/>
+      <c r="Z2" s="41"/>
+      <c r="AA2" s="41"/>
+      <c r="AB2" s="41"/>
+      <c r="AC2" s="41"/>
+      <c r="AD2" s="41"/>
+      <c r="AE2" s="41"/>
+      <c r="AF2" s="41"/>
+      <c r="AG2" s="41"/>
+      <c r="AH2" s="41"/>
+      <c r="AI2" s="41"/>
+      <c r="AJ2" s="41"/>
+      <c r="AK2" s="41"/>
+      <c r="AL2" s="41"/>
+      <c r="AM2" s="41"/>
+      <c r="AN2" s="41"/>
+      <c r="AO2" s="41"/>
+      <c r="AP2" s="41"/>
+      <c r="AQ2" s="41"/>
+      <c r="AR2" s="41"/>
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="42" t="s">
         <v>272</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="39" t="s">
+      <c r="E3" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="39" t="s">
+      <c r="F3" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="39" t="s">
+      <c r="G3" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="39" t="s">
+      <c r="H3" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="39" t="s">
+      <c r="I3" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="39" t="s">
+      <c r="J3" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="39" t="s">
+      <c r="K3" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="39" t="s">
+      <c r="L3" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="40"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="40"/>
-      <c r="V3" s="40"/>
-      <c r="W3" s="40"/>
-      <c r="X3" s="40"/>
-      <c r="Y3" s="40"/>
-      <c r="Z3" s="40"/>
-      <c r="AA3" s="40"/>
-      <c r="AB3" s="40"/>
-      <c r="AC3" s="40"/>
-      <c r="AD3" s="40"/>
-      <c r="AE3" s="40"/>
-      <c r="AF3" s="40"/>
-      <c r="AG3" s="40"/>
-      <c r="AH3" s="40"/>
-      <c r="AI3" s="40"/>
-      <c r="AJ3" s="40"/>
-      <c r="AK3" s="40"/>
-      <c r="AL3" s="40"/>
-      <c r="AM3" s="40"/>
-      <c r="AN3" s="40"/>
-      <c r="AO3" s="40"/>
-      <c r="AP3" s="40"/>
-      <c r="AQ3" s="40"/>
-      <c r="AR3" s="40"/>
+      <c r="M3" s="41"/>
+      <c r="N3" s="41"/>
+      <c r="O3" s="41"/>
+      <c r="P3" s="41"/>
+      <c r="Q3" s="41"/>
+      <c r="R3" s="41"/>
+      <c r="S3" s="41"/>
+      <c r="T3" s="41"/>
+      <c r="U3" s="41"/>
+      <c r="V3" s="41"/>
+      <c r="W3" s="41"/>
+      <c r="X3" s="41"/>
+      <c r="Y3" s="41"/>
+      <c r="Z3" s="41"/>
+      <c r="AA3" s="41"/>
+      <c r="AB3" s="41"/>
+      <c r="AC3" s="41"/>
+      <c r="AD3" s="41"/>
+      <c r="AE3" s="41"/>
+      <c r="AF3" s="41"/>
+      <c r="AG3" s="41"/>
+      <c r="AH3" s="41"/>
+      <c r="AI3" s="41"/>
+      <c r="AJ3" s="41"/>
+      <c r="AK3" s="41"/>
+      <c r="AL3" s="41"/>
+      <c r="AM3" s="41"/>
+      <c r="AN3" s="41"/>
+      <c r="AO3" s="41"/>
+      <c r="AP3" s="41"/>
+      <c r="AQ3" s="41"/>
+      <c r="AR3" s="41"/>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="42" t="s">
         <v>273</v>
       </c>
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="39" t="s">
+      <c r="E4" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="39" t="s">
+      <c r="F4" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="G4" s="39" t="s">
+      <c r="G4" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="40"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="40"/>
-      <c r="K4" s="40"/>
-      <c r="L4" s="40"/>
-      <c r="M4" s="40"/>
-      <c r="N4" s="40"/>
-      <c r="O4" s="40"/>
-      <c r="P4" s="40"/>
-      <c r="Q4" s="40"/>
-      <c r="R4" s="40"/>
-      <c r="S4" s="40"/>
-      <c r="T4" s="40"/>
-      <c r="U4" s="40"/>
-      <c r="V4" s="40"/>
-      <c r="W4" s="40"/>
-      <c r="X4" s="40"/>
-      <c r="Y4" s="40"/>
-      <c r="Z4" s="40"/>
-      <c r="AA4" s="40"/>
-      <c r="AB4" s="40"/>
-      <c r="AC4" s="40"/>
-      <c r="AD4" s="40"/>
-      <c r="AE4" s="40"/>
-      <c r="AF4" s="40"/>
-      <c r="AG4" s="40"/>
-      <c r="AH4" s="40"/>
-      <c r="AI4" s="40"/>
-      <c r="AJ4" s="40"/>
-      <c r="AK4" s="40"/>
-      <c r="AL4" s="40"/>
-      <c r="AM4" s="40"/>
-      <c r="AN4" s="40"/>
-      <c r="AO4" s="40"/>
-      <c r="AP4" s="40"/>
-      <c r="AQ4" s="40"/>
-      <c r="AR4" s="40"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="41"/>
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="41"/>
+      <c r="V4" s="41"/>
+      <c r="W4" s="41"/>
+      <c r="X4" s="41"/>
+      <c r="Y4" s="41"/>
+      <c r="Z4" s="41"/>
+      <c r="AA4" s="41"/>
+      <c r="AB4" s="41"/>
+      <c r="AC4" s="41"/>
+      <c r="AD4" s="41"/>
+      <c r="AE4" s="41"/>
+      <c r="AF4" s="41"/>
+      <c r="AG4" s="41"/>
+      <c r="AH4" s="41"/>
+      <c r="AI4" s="41"/>
+      <c r="AJ4" s="41"/>
+      <c r="AK4" s="41"/>
+      <c r="AL4" s="41"/>
+      <c r="AM4" s="41"/>
+      <c r="AN4" s="41"/>
+      <c r="AO4" s="41"/>
+      <c r="AP4" s="41"/>
+      <c r="AQ4" s="41"/>
+      <c r="AR4" s="41"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="42" t="s">
         <v>274</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="40"/>
-      <c r="K5" s="40"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="40"/>
-      <c r="N5" s="40"/>
-      <c r="O5" s="40"/>
-      <c r="P5" s="40"/>
-      <c r="Q5" s="40"/>
-      <c r="R5" s="40"/>
-      <c r="S5" s="40"/>
-      <c r="T5" s="40"/>
-      <c r="U5" s="40"/>
-      <c r="V5" s="40"/>
-      <c r="W5" s="40"/>
-      <c r="X5" s="40"/>
-      <c r="Y5" s="40"/>
-      <c r="Z5" s="40"/>
-      <c r="AA5" s="40"/>
-      <c r="AB5" s="40"/>
-      <c r="AC5" s="40"/>
-      <c r="AD5" s="40"/>
-      <c r="AE5" s="40"/>
-      <c r="AF5" s="40"/>
-      <c r="AG5" s="40"/>
-      <c r="AH5" s="40"/>
-      <c r="AI5" s="40"/>
-      <c r="AJ5" s="40"/>
-      <c r="AK5" s="40"/>
-      <c r="AL5" s="40"/>
-      <c r="AM5" s="40"/>
-      <c r="AN5" s="40"/>
-      <c r="AO5" s="40"/>
-      <c r="AP5" s="40"/>
-      <c r="AQ5" s="40"/>
-      <c r="AR5" s="40"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="41"/>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="41"/>
+      <c r="R5" s="41"/>
+      <c r="S5" s="41"/>
+      <c r="T5" s="41"/>
+      <c r="U5" s="41"/>
+      <c r="V5" s="41"/>
+      <c r="W5" s="41"/>
+      <c r="X5" s="41"/>
+      <c r="Y5" s="41"/>
+      <c r="Z5" s="41"/>
+      <c r="AA5" s="41"/>
+      <c r="AB5" s="41"/>
+      <c r="AC5" s="41"/>
+      <c r="AD5" s="41"/>
+      <c r="AE5" s="41"/>
+      <c r="AF5" s="41"/>
+      <c r="AG5" s="41"/>
+      <c r="AH5" s="41"/>
+      <c r="AI5" s="41"/>
+      <c r="AJ5" s="41"/>
+      <c r="AK5" s="41"/>
+      <c r="AL5" s="41"/>
+      <c r="AM5" s="41"/>
+      <c r="AN5" s="41"/>
+      <c r="AO5" s="41"/>
+      <c r="AP5" s="41"/>
+      <c r="AQ5" s="41"/>
+      <c r="AR5" s="41"/>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="42" t="s">
         <v>275</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="40" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="40" t="s">
         <v>118</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="40" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="39" t="s">
+      <c r="E6" s="40" t="s">
         <v>122</v>
       </c>
-      <c r="F6" s="39" t="s">
+      <c r="F6" s="40" t="s">
         <v>124</v>
       </c>
-      <c r="G6" s="39" t="s">
+      <c r="G6" s="40" t="s">
         <v>126</v>
       </c>
-      <c r="H6" s="39" t="s">
+      <c r="H6" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="I6" s="39" t="s">
+      <c r="I6" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="J6" s="39" t="s">
+      <c r="J6" s="40" t="s">
         <v>132</v>
       </c>
-      <c r="K6" s="39" t="s">
+      <c r="K6" s="40" t="s">
         <v>134</v>
       </c>
-      <c r="L6" s="39" t="s">
+      <c r="L6" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="M6" s="39" t="s">
+      <c r="M6" s="40" t="s">
         <v>139</v>
       </c>
-      <c r="N6" s="39" t="s">
+      <c r="N6" s="40" t="s">
         <v>141</v>
       </c>
-      <c r="O6" s="39" t="s">
+      <c r="O6" s="40" t="s">
         <v>143</v>
       </c>
-      <c r="P6" s="39" t="s">
+      <c r="P6" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="Q6" s="39" t="s">
+      <c r="Q6" s="40" t="s">
         <v>147</v>
       </c>
-      <c r="R6" s="39" t="s">
+      <c r="R6" s="40" t="s">
         <v>149</v>
       </c>
-      <c r="S6" s="39" t="s">
+      <c r="S6" s="40" t="s">
         <v>151</v>
       </c>
-      <c r="T6" s="39" t="s">
+      <c r="T6" s="40" t="s">
         <v>153</v>
       </c>
-      <c r="U6" s="39" t="s">
+      <c r="U6" s="40" t="s">
         <v>155</v>
       </c>
-      <c r="V6" s="39" t="s">
+      <c r="V6" s="40" t="s">
         <v>157</v>
       </c>
-      <c r="W6" s="39" t="s">
+      <c r="W6" s="40" t="s">
         <v>159</v>
       </c>
-      <c r="X6" s="39" t="s">
+      <c r="X6" s="40" t="s">
         <v>161</v>
       </c>
-      <c r="Y6" s="39" t="s">
+      <c r="Y6" s="40" t="s">
         <v>163</v>
       </c>
-      <c r="Z6" s="39" t="s">
+      <c r="Z6" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="AA6" s="39" t="s">
+      <c r="AA6" s="40" t="s">
         <v>167</v>
       </c>
-      <c r="AB6" s="39" t="s">
+      <c r="AB6" s="40" t="s">
         <v>169</v>
       </c>
-      <c r="AC6" s="39" t="s">
+      <c r="AC6" s="40" t="s">
         <v>171</v>
       </c>
-      <c r="AD6" s="39" t="s">
+      <c r="AD6" s="40" t="s">
         <v>173</v>
       </c>
-      <c r="AE6" s="39" t="s">
+      <c r="AE6" s="40" t="s">
         <v>175</v>
       </c>
-      <c r="AF6" s="39" t="s">
+      <c r="AF6" s="40" t="s">
         <v>177</v>
       </c>
-      <c r="AG6" s="39" t="s">
+      <c r="AG6" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="AH6" s="39" t="s">
+      <c r="AH6" s="40" t="s">
         <v>181</v>
       </c>
-      <c r="AI6" s="39" t="s">
+      <c r="AI6" s="40" t="s">
         <v>183</v>
       </c>
-      <c r="AJ6" s="39" t="s">
+      <c r="AJ6" s="40" t="s">
         <v>185</v>
       </c>
-      <c r="AK6" s="39" t="s">
+      <c r="AK6" s="40" t="s">
         <v>187</v>
       </c>
-      <c r="AL6" s="39" t="s">
+      <c r="AL6" s="40" t="s">
         <v>189</v>
       </c>
-      <c r="AM6" s="39" t="s">
+      <c r="AM6" s="40" t="s">
         <v>191</v>
       </c>
-      <c r="AN6" s="39" t="s">
+      <c r="AN6" s="40" t="s">
         <v>193</v>
       </c>
-      <c r="AO6" s="39" t="s">
+      <c r="AO6" s="40" t="s">
         <v>196</v>
       </c>
-      <c r="AP6" s="39" t="s">
+      <c r="AP6" s="40" t="s">
         <v>198</v>
       </c>
-      <c r="AQ6" s="39" t="s">
+      <c r="AQ6" s="40" t="s">
         <v>200</v>
       </c>
-      <c r="AR6" s="39" t="s">
+      <c r="AR6" s="40" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="43" t="s">
         <v>276</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="40" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="40" t="s">
         <v>118</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="D7" s="40" t="s">
         <v>120</v>
       </c>
-      <c r="E7" s="39" t="s">
+      <c r="E7" s="40" t="s">
         <v>122</v>
       </c>
-      <c r="F7" s="39" t="s">
+      <c r="F7" s="40" t="s">
         <v>124</v>
       </c>
-      <c r="G7" s="39" t="s">
+      <c r="G7" s="40" t="s">
         <v>126</v>
       </c>
-      <c r="H7" s="39" t="s">
+      <c r="H7" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="I7" s="39" t="s">
+      <c r="I7" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="J7" s="39" t="s">
+      <c r="J7" s="40" t="s">
         <v>132</v>
       </c>
-      <c r="K7" s="39" t="s">
+      <c r="K7" s="40" t="s">
         <v>134</v>
       </c>
-      <c r="L7" s="39" t="s">
+      <c r="L7" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="M7" s="39" t="s">
+      <c r="M7" s="40" t="s">
         <v>147</v>
       </c>
-      <c r="N7" s="39" t="s">
+      <c r="N7" s="40" t="s">
         <v>149</v>
       </c>
-      <c r="O7" s="39" t="s">
+      <c r="O7" s="40" t="s">
         <v>151</v>
       </c>
-      <c r="P7" s="39" t="s">
+      <c r="P7" s="40" t="s">
         <v>153</v>
       </c>
-      <c r="Q7" s="39" t="s">
+      <c r="Q7" s="40" t="s">
         <v>155</v>
       </c>
-      <c r="R7" s="39" t="s">
+      <c r="R7" s="40" t="s">
         <v>157</v>
       </c>
-      <c r="S7" s="39" t="s">
+      <c r="S7" s="40" t="s">
         <v>159</v>
       </c>
-      <c r="T7" s="39" t="s">
+      <c r="T7" s="40" t="s">
         <v>161</v>
       </c>
-      <c r="U7" s="39" t="s">
+      <c r="U7" s="40" t="s">
         <v>163</v>
       </c>
-      <c r="V7" s="39" t="s">
+      <c r="V7" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="W7" s="39" t="s">
+      <c r="W7" s="40" t="s">
         <v>167</v>
       </c>
-      <c r="X7" s="39" t="s">
+      <c r="X7" s="40" t="s">
         <v>169</v>
       </c>
-      <c r="Y7" s="39" t="s">
+      <c r="Y7" s="40" t="s">
         <v>171</v>
       </c>
-      <c r="Z7" s="39" t="s">
+      <c r="Z7" s="40" t="s">
         <v>173</v>
       </c>
-      <c r="AA7" s="39" t="s">
+      <c r="AA7" s="40" t="s">
         <v>175</v>
       </c>
-      <c r="AB7" s="39" t="s">
+      <c r="AB7" s="40" t="s">
         <v>177</v>
       </c>
-      <c r="AC7" s="39" t="s">
+      <c r="AC7" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="AD7" s="39" t="s">
+      <c r="AD7" s="40" t="s">
         <v>181</v>
       </c>
-      <c r="AE7" s="39" t="s">
+      <c r="AE7" s="40" t="s">
         <v>183</v>
       </c>
-      <c r="AF7" s="39" t="s">
+      <c r="AF7" s="40" t="s">
         <v>185</v>
       </c>
-      <c r="AG7" s="39" t="s">
+      <c r="AG7" s="40" t="s">
         <v>187</v>
       </c>
-      <c r="AH7" s="39" t="s">
+      <c r="AH7" s="40" t="s">
         <v>189</v>
       </c>
-      <c r="AI7" s="39" t="s">
+      <c r="AI7" s="40" t="s">
         <v>191</v>
       </c>
-      <c r="AJ7" s="40"/>
-      <c r="AK7" s="40"/>
-      <c r="AL7" s="40"/>
-      <c r="AM7" s="40"/>
-      <c r="AN7" s="40"/>
-      <c r="AO7" s="40"/>
-      <c r="AP7" s="40"/>
-      <c r="AQ7" s="40"/>
-      <c r="AR7" s="40"/>
+      <c r="AJ7" s="41"/>
+      <c r="AK7" s="41"/>
+      <c r="AL7" s="41"/>
+      <c r="AM7" s="41"/>
+      <c r="AN7" s="41"/>
+      <c r="AO7" s="41"/>
+      <c r="AP7" s="41"/>
+      <c r="AQ7" s="41"/>
+      <c r="AR7" s="41"/>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="43" t="s">
         <v>277</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="40" t="s">
         <v>215</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="C8" s="40" t="s">
         <v>217</v>
       </c>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="40"/>
-      <c r="K8" s="40"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="40"/>
-      <c r="N8" s="40"/>
-      <c r="O8" s="40"/>
-      <c r="P8" s="40"/>
-      <c r="Q8" s="40"/>
-      <c r="R8" s="40"/>
-      <c r="S8" s="40"/>
-      <c r="T8" s="40"/>
-      <c r="U8" s="40"/>
-      <c r="V8" s="40"/>
-      <c r="W8" s="40"/>
-      <c r="X8" s="40"/>
-      <c r="Y8" s="40"/>
-      <c r="Z8" s="40"/>
-      <c r="AA8" s="40"/>
-      <c r="AB8" s="40"/>
-      <c r="AC8" s="40"/>
-      <c r="AD8" s="40"/>
-      <c r="AE8" s="40"/>
-      <c r="AF8" s="40"/>
-      <c r="AG8" s="40"/>
-      <c r="AH8" s="40"/>
-      <c r="AI8" s="40"/>
-      <c r="AJ8" s="40"/>
-      <c r="AK8" s="40"/>
-      <c r="AL8" s="40"/>
-      <c r="AM8" s="40"/>
-      <c r="AN8" s="40"/>
-      <c r="AO8" s="40"/>
-      <c r="AP8" s="40"/>
-      <c r="AQ8" s="40"/>
-      <c r="AR8" s="40"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="41"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="41"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="41"/>
+      <c r="O8" s="41"/>
+      <c r="P8" s="41"/>
+      <c r="Q8" s="41"/>
+      <c r="R8" s="41"/>
+      <c r="S8" s="41"/>
+      <c r="T8" s="41"/>
+      <c r="U8" s="41"/>
+      <c r="V8" s="41"/>
+      <c r="W8" s="41"/>
+      <c r="X8" s="41"/>
+      <c r="Y8" s="41"/>
+      <c r="Z8" s="41"/>
+      <c r="AA8" s="41"/>
+      <c r="AB8" s="41"/>
+      <c r="AC8" s="41"/>
+      <c r="AD8" s="41"/>
+      <c r="AE8" s="41"/>
+      <c r="AF8" s="41"/>
+      <c r="AG8" s="41"/>
+      <c r="AH8" s="41"/>
+      <c r="AI8" s="41"/>
+      <c r="AJ8" s="41"/>
+      <c r="AK8" s="41"/>
+      <c r="AL8" s="41"/>
+      <c r="AM8" s="41"/>
+      <c r="AN8" s="41"/>
+      <c r="AO8" s="41"/>
+      <c r="AP8" s="41"/>
+      <c r="AQ8" s="41"/>
+      <c r="AR8" s="41"/>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="43" t="s">
         <v>278</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="40" t="s">
         <v>215</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="40" t="s">
         <v>217</v>
       </c>
-      <c r="D9" s="44" t="s">
+      <c r="D9" s="48" t="s">
         <v>285</v>
       </c>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="40"/>
-      <c r="I9" s="40"/>
-      <c r="J9" s="40"/>
-      <c r="K9" s="40"/>
-      <c r="L9" s="40"/>
-      <c r="M9" s="40"/>
-      <c r="N9" s="40"/>
-      <c r="O9" s="40"/>
-      <c r="P9" s="40"/>
-      <c r="Q9" s="40"/>
-      <c r="R9" s="40"/>
-      <c r="S9" s="40"/>
-      <c r="T9" s="40"/>
-      <c r="U9" s="40"/>
-      <c r="V9" s="40"/>
-      <c r="W9" s="40"/>
-      <c r="X9" s="40"/>
-      <c r="Y9" s="40"/>
-      <c r="Z9" s="40"/>
-      <c r="AA9" s="40"/>
-      <c r="AB9" s="40"/>
-      <c r="AC9" s="40"/>
-      <c r="AD9" s="40"/>
-      <c r="AE9" s="40"/>
-      <c r="AF9" s="40"/>
-      <c r="AG9" s="40"/>
-      <c r="AH9" s="40"/>
-      <c r="AI9" s="40"/>
-      <c r="AJ9" s="40"/>
-      <c r="AK9" s="40"/>
-      <c r="AL9" s="40"/>
-      <c r="AM9" s="40"/>
-      <c r="AN9" s="40"/>
-      <c r="AO9" s="40"/>
-      <c r="AP9" s="40"/>
-      <c r="AQ9" s="40"/>
-      <c r="AR9" s="40"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="41"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="41"/>
+      <c r="M9" s="41"/>
+      <c r="N9" s="41"/>
+      <c r="O9" s="41"/>
+      <c r="P9" s="41"/>
+      <c r="Q9" s="41"/>
+      <c r="R9" s="41"/>
+      <c r="S9" s="41"/>
+      <c r="T9" s="41"/>
+      <c r="U9" s="41"/>
+      <c r="V9" s="41"/>
+      <c r="W9" s="41"/>
+      <c r="X9" s="41"/>
+      <c r="Y9" s="41"/>
+      <c r="Z9" s="41"/>
+      <c r="AA9" s="41"/>
+      <c r="AB9" s="41"/>
+      <c r="AC9" s="41"/>
+      <c r="AD9" s="41"/>
+      <c r="AE9" s="41"/>
+      <c r="AF9" s="41"/>
+      <c r="AG9" s="41"/>
+      <c r="AH9" s="41"/>
+      <c r="AI9" s="41"/>
+      <c r="AJ9" s="41"/>
+      <c r="AK9" s="41"/>
+      <c r="AL9" s="41"/>
+      <c r="AM9" s="41"/>
+      <c r="AN9" s="41"/>
+      <c r="AO9" s="41"/>
+      <c r="AP9" s="41"/>
+      <c r="AQ9" s="41"/>
+      <c r="AR9" s="41"/>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="43" t="s">
         <v>279</v>
       </c>
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="40" t="s">
         <v>219</v>
       </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="40"/>
-      <c r="K10" s="40"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="40"/>
-      <c r="N10" s="40"/>
-      <c r="O10" s="40"/>
-      <c r="P10" s="40"/>
-      <c r="Q10" s="40"/>
-      <c r="R10" s="40"/>
-      <c r="S10" s="40"/>
-      <c r="T10" s="40"/>
-      <c r="U10" s="40"/>
-      <c r="V10" s="40"/>
-      <c r="W10" s="40"/>
-      <c r="X10" s="40"/>
-      <c r="Y10" s="40"/>
-      <c r="Z10" s="40"/>
-      <c r="AA10" s="40"/>
-      <c r="AB10" s="40"/>
-      <c r="AC10" s="40"/>
-      <c r="AD10" s="40"/>
-      <c r="AE10" s="40"/>
-      <c r="AF10" s="40"/>
-      <c r="AG10" s="40"/>
-      <c r="AH10" s="40"/>
-      <c r="AI10" s="40"/>
-      <c r="AJ10" s="40"/>
-      <c r="AK10" s="40"/>
-      <c r="AL10" s="40"/>
-      <c r="AM10" s="40"/>
-      <c r="AN10" s="40"/>
-      <c r="AO10" s="40"/>
-      <c r="AP10" s="40"/>
-      <c r="AQ10" s="40"/>
-      <c r="AR10" s="40"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="41"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="41"/>
+      <c r="P10" s="41"/>
+      <c r="Q10" s="41"/>
+      <c r="R10" s="41"/>
+      <c r="S10" s="41"/>
+      <c r="T10" s="41"/>
+      <c r="U10" s="41"/>
+      <c r="V10" s="41"/>
+      <c r="W10" s="41"/>
+      <c r="X10" s="41"/>
+      <c r="Y10" s="41"/>
+      <c r="Z10" s="41"/>
+      <c r="AA10" s="41"/>
+      <c r="AB10" s="41"/>
+      <c r="AC10" s="41"/>
+      <c r="AD10" s="41"/>
+      <c r="AE10" s="41"/>
+      <c r="AF10" s="41"/>
+      <c r="AG10" s="41"/>
+      <c r="AH10" s="41"/>
+      <c r="AI10" s="41"/>
+      <c r="AJ10" s="41"/>
+      <c r="AK10" s="41"/>
+      <c r="AL10" s="41"/>
+      <c r="AM10" s="41"/>
+      <c r="AN10" s="41"/>
+      <c r="AO10" s="41"/>
+      <c r="AP10" s="41"/>
+      <c r="AQ10" s="41"/>
+      <c r="AR10" s="41"/>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="43" t="s">
         <v>280</v>
       </c>
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="40" t="s">
         <v>204</v>
       </c>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="40"/>
-      <c r="J11" s="40"/>
-      <c r="K11" s="40"/>
-      <c r="L11" s="40"/>
-      <c r="M11" s="40"/>
-      <c r="N11" s="40"/>
-      <c r="O11" s="40"/>
-      <c r="P11" s="40"/>
-      <c r="Q11" s="40"/>
-      <c r="R11" s="40"/>
-      <c r="S11" s="40"/>
-      <c r="T11" s="40"/>
-      <c r="U11" s="40"/>
-      <c r="V11" s="40"/>
-      <c r="W11" s="40"/>
-      <c r="X11" s="40"/>
-      <c r="Y11" s="40"/>
-      <c r="Z11" s="40"/>
-      <c r="AA11" s="40"/>
-      <c r="AB11" s="40"/>
-      <c r="AC11" s="40"/>
-      <c r="AD11" s="40"/>
-      <c r="AE11" s="40"/>
-      <c r="AF11" s="40"/>
-      <c r="AG11" s="40"/>
-      <c r="AH11" s="40"/>
-      <c r="AI11" s="40"/>
-      <c r="AJ11" s="40"/>
-      <c r="AK11" s="40"/>
-      <c r="AL11" s="40"/>
-      <c r="AM11" s="40"/>
-      <c r="AN11" s="40"/>
-      <c r="AO11" s="40"/>
-      <c r="AP11" s="40"/>
-      <c r="AQ11" s="40"/>
-      <c r="AR11" s="40"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="41"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+      <c r="M11" s="41"/>
+      <c r="N11" s="41"/>
+      <c r="O11" s="41"/>
+      <c r="P11" s="41"/>
+      <c r="Q11" s="41"/>
+      <c r="R11" s="41"/>
+      <c r="S11" s="41"/>
+      <c r="T11" s="41"/>
+      <c r="U11" s="41"/>
+      <c r="V11" s="41"/>
+      <c r="W11" s="41"/>
+      <c r="X11" s="41"/>
+      <c r="Y11" s="41"/>
+      <c r="Z11" s="41"/>
+      <c r="AA11" s="41"/>
+      <c r="AB11" s="41"/>
+      <c r="AC11" s="41"/>
+      <c r="AD11" s="41"/>
+      <c r="AE11" s="41"/>
+      <c r="AF11" s="41"/>
+      <c r="AG11" s="41"/>
+      <c r="AH11" s="41"/>
+      <c r="AI11" s="41"/>
+      <c r="AJ11" s="41"/>
+      <c r="AK11" s="41"/>
+      <c r="AL11" s="41"/>
+      <c r="AM11" s="41"/>
+      <c r="AN11" s="41"/>
+      <c r="AO11" s="41"/>
+      <c r="AP11" s="41"/>
+      <c r="AQ11" s="41"/>
+      <c r="AR11" s="41"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>